<commit_message>
refactor: improve project document handling with timeline parsing, template configuration, and robust replacement logic
</commit_message>
<xml_diff>
--- a/Form checklist hồ sơ dự án.xlsx
+++ b/Form checklist hồ sơ dự án.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Đề tài - Bánh ăn dặm VIAM 2027" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Đề tài - Mẫu trắng dự án mới" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đề tài - Bánh ăn dặm VIAM 2027" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đề tài - Mẫu trắng dự án mới" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Arial"/>
       <family val="2"/>
@@ -56,6 +56,9 @@
       <color indexed="9"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="6">
@@ -102,13 +105,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1988,7 +1992,7 @@
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Lý lịch khoa học-TruongHongSon.doc</t>
+          <t>Lý lịch khoa học - Trương Hồng Sơn.docx</t>
         </is>
       </c>
       <c r="F67">

</xml_diff>

<commit_message>
feat: add optional checklist field A07 for research location
</commit_message>
<xml_diff>
--- a/Form checklist hồ sơ dự án.xlsx
+++ b/Form checklist hồ sơ dự án.xlsx
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F76"/>
+  <dimension ref="A1:F77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="8.5" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -715,92 +715,80 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>A07</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Địa điểm triển khai nghiên cứu (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n"/>
+      <c r="D12" s="3" t="n"/>
+      <c r="E12" s="3" t="n"/>
+      <c r="F12">
+        <f>IF(ISBLANK(C12), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>SEC_B</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>PHẦN B: BAN CHỦ NHIỆM &amp; NGHIÊN CỨU VIÊN ĐỀ TÀI (TỐI ĐA 20 NGƯỜI)</t>
         </is>
       </c>
-      <c r="C12" s="2" t="n"/>
-      <c r="D12" s="2" t="n"/>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>B01</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Chủ nhiệm đề tài (CNĐT - Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Trương Hồng Sơn</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>TS.BS.</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>Viện trưởng - Viện Y học Ứng dụng VN</t>
-        </is>
-      </c>
-      <c r="F13">
-        <f>IF(ISBLANK(C13), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
-        <v/>
-      </c>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>B02</t>
+          <t>B01</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Đồng Chủ nhiệm đề tài (Tùy chọn)</t>
+          <t>Chủ nhiệm đề tài (CNĐT - Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Trương Hồng Sơn</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>TS.BS.</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Viện trưởng - Viện Y học Ứng dụng VN</t>
         </is>
       </c>
       <c r="F14">
-        <f>IF(ISBLANK(C14), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C14), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>B03</t>
+          <t>B02</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Thư ký Đề tài (Khác Thư ký HĐ - Tùy chọn)</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Lưu Liên Hương</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Thạc sĩ</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Trung tâm NCKH - Viện VIAM</t>
+          <t>Đồng Chủ nhiệm đề tài (Tùy chọn)</t>
         </is>
       </c>
       <c r="F15">
@@ -811,17 +799,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>B04</t>
+          <t>B03</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 1</t>
+          <t>Thư ký Đề tài (Khác Thư ký HĐ - Tùy chọn)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Lê Việt Anh</t>
+          <t>Lưu Liên Hương</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -842,27 +830,27 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>B05</t>
+          <t>B04</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 2</t>
+          <t>Nghiên cứu viên 1</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Lê Minh Khánh</t>
+          <t>Lê Việt Anh</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Bác sĩ</t>
+          <t>Thạc sĩ</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Phòng khám VIAM</t>
+          <t>Trung tâm NCKH - Viện VIAM</t>
         </is>
       </c>
       <c r="F17">
@@ -873,12 +861,27 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>B06</t>
+          <t>B05</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 3</t>
+          <t>Nghiên cứu viên 2</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Lê Minh Khánh</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Bác sĩ</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Phòng khám VIAM</t>
         </is>
       </c>
       <c r="F18">
@@ -889,12 +892,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>B07</t>
+          <t>B06</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 4</t>
+          <t>Nghiên cứu viên 3</t>
         </is>
       </c>
       <c r="F19">
@@ -905,12 +908,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>B08</t>
+          <t>B07</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 5</t>
+          <t>Nghiên cứu viên 4</t>
         </is>
       </c>
       <c r="F20">
@@ -921,12 +924,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>B09</t>
+          <t>B08</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 6</t>
+          <t>Nghiên cứu viên 5</t>
         </is>
       </c>
       <c r="F21">
@@ -937,12 +940,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>B10</t>
+          <t>B09</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 7</t>
+          <t>Nghiên cứu viên 6</t>
         </is>
       </c>
       <c r="F22">
@@ -953,12 +956,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>B11</t>
+          <t>B10</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 8</t>
+          <t>Nghiên cứu viên 7</t>
         </is>
       </c>
       <c r="F23">
@@ -969,12 +972,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>B12</t>
+          <t>B11</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 9</t>
+          <t>Nghiên cứu viên 8</t>
         </is>
       </c>
       <c r="F24">
@@ -985,12 +988,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>B13</t>
+          <t>B12</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 10</t>
+          <t>Nghiên cứu viên 9</t>
         </is>
       </c>
       <c r="F25">
@@ -1001,12 +1004,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>B14</t>
+          <t>B13</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 11</t>
+          <t>Nghiên cứu viên 10</t>
         </is>
       </c>
       <c r="F26">
@@ -1017,12 +1020,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>B15</t>
+          <t>B14</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 12</t>
+          <t>Nghiên cứu viên 11</t>
         </is>
       </c>
       <c r="F27">
@@ -1033,12 +1036,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>B16</t>
+          <t>B15</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 13</t>
+          <t>Nghiên cứu viên 12</t>
         </is>
       </c>
       <c r="F28">
@@ -1049,12 +1052,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>B17</t>
+          <t>B16</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 14</t>
+          <t>Nghiên cứu viên 13</t>
         </is>
       </c>
       <c r="F29">
@@ -1065,12 +1068,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>B18</t>
+          <t>B17</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 15</t>
+          <t>Nghiên cứu viên 14</t>
         </is>
       </c>
       <c r="F30">
@@ -1081,12 +1084,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>B19</t>
+          <t>B18</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 16</t>
+          <t>Nghiên cứu viên 15</t>
         </is>
       </c>
       <c r="F31">
@@ -1097,12 +1100,12 @@
     <row r="32" ht="15" customHeight="1">
       <c r="A32" t="inlineStr">
         <is>
-          <t>B20</t>
+          <t>B19</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 17</t>
+          <t>Nghiên cứu viên 16</t>
         </is>
       </c>
       <c r="F32">
@@ -1111,76 +1114,61 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>B20</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Nghiên cứu viên 17</t>
+        </is>
+      </c>
+      <c r="F33">
+        <f>IF(ISBLANK(C33), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>SEC_C</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>PHẦN C: HỘI ĐỒNG ĐẠO ĐỨC TRONG NGHIÊN CỨU (HĐ 01 - 7 THÀNH VIÊN BẮT BUỘC)</t>
         </is>
       </c>
-      <c r="C33" s="2" t="n"/>
-      <c r="D33" s="2" t="n"/>
-      <c r="E33" s="2" t="n"/>
-      <c r="F33" s="2" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>C01</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Chủ tịch HĐ Đạo đức (Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>Nguyễn Công Khẩn</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>GS.TS.</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr">
-        <is>
-          <t>Hội đồng Đạo đức Y sinh Quốc gia</t>
-        </is>
-      </c>
-      <c r="F34">
-        <f>IF(ISBLANK(C34), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
-        <v/>
-      </c>
+      <c r="C34" s="2" t="n"/>
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>C02</t>
+          <t>C01</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 1 (Bắt buộc)</t>
+          <t>Chủ tịch HĐ Đạo đức (Bắt buộc)</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Xuân Ninh</t>
+          <t>Nguyễn Công Khẩn</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>PGS.TS.BS.</t>
+          <t>GS.TS.</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Viện Y học Ứng dụng Việt Nam</t>
+          <t>Hội đồng Đạo đức Y sinh Quốc gia</t>
         </is>
       </c>
       <c r="F35">
@@ -1191,17 +1179,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>C03</t>
+          <t>C02</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 2 (Bắt buộc)</t>
+          <t>Ủy viên Phản biện 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Lê Bạch Mai</t>
+          <t>Nguyễn Xuân Ninh</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -1211,7 +1199,7 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Nguyên Phó Viện trưởng Viện Dinh dưỡng QG</t>
+          <t>Viện Y học Ứng dụng Việt Nam</t>
         </is>
       </c>
       <c r="F36">
@@ -1222,17 +1210,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>C04</t>
+          <t>C03</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đạo đức 1 (Bắt buộc)</t>
+          <t>Ủy viên Phản biện 2 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Thị Lâm</t>
+          <t>Lê Bạch Mai</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -1253,17 +1241,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>C05</t>
+          <t>C04</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đạo đức 2 (Bắt buộc)</t>
+          <t>Ủy viên HĐ Đạo đức 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Quang Dũng</t>
+          <t>Nguyễn Thị Lâm</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -1273,7 +1261,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Bộ môn Dinh dưỡng - ĐH Y Hà Nội</t>
+          <t>Nguyên Phó Viện trưởng Viện Dinh dưỡng QG</t>
         </is>
       </c>
       <c r="F38">
@@ -1284,28 +1272,43 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>C06</t>
+          <t>C05</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 3 (Tùy chọn)</t>
+          <t>Ủy viên HĐ Đạo đức 2 (Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Nguyễn Quang Dũng</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>PGS.TS.BS.</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Bộ môn Dinh dưỡng - ĐH Y Hà Nội</t>
         </is>
       </c>
       <c r="F39">
-        <f>IF(ISBLANK(C39), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C39), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>C07</t>
+          <t>C06</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đạo đức 3 (Tùy chọn)</t>
+          <t>Ủy viên Phản biện 3 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F40">
@@ -1316,12 +1319,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>C08</t>
+          <t>C07</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đạo đức 4 (Tùy chọn)</t>
+          <t>Ủy viên HĐ Đạo đức 3 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F41">
@@ -1332,48 +1335,33 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>C09</t>
+          <t>C08</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Thư ký HĐ Đạo đức 1 (Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>Hoàng Hà Linh</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>Thạc sĩ</t>
-        </is>
-      </c>
-      <c r="E42" s="3" t="inlineStr">
-        <is>
-          <t>Trung tâm NCKH - Viện VIAM</t>
+          <t>Ủy viên HĐ Đạo đức 4 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F42">
-        <f>IF(ISBLANK(C42), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C42), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" t="inlineStr">
         <is>
-          <t>C10</t>
+          <t>C09</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Thư ký HĐ Đạo đức 2 (Bắt buộc)</t>
+          <t>Thư ký HĐ Đạo đức 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Trương Phan Hồng Hà</t>
+          <t>Hoàng Hà Linh</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -1383,7 +1371,7 @@
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Viện Y học Ứng dụng Việt Nam</t>
+          <t>Trung tâm NCKH - Viện VIAM</t>
         </is>
       </c>
       <c r="F43">
@@ -1392,76 +1380,76 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Thư ký HĐ Đạo đức 2 (Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Trương Phan Hồng Hà</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Thạc sĩ</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Viện Y học Ứng dụng Việt Nam</t>
+        </is>
+      </c>
+      <c r="F44">
+        <f>IF(ISBLANK(C44), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>SEC_D</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>PHẦN D: HỘI ĐỒNG KHOA HỌC XÉT DUYỆT ĐỀ CƯƠNG (HĐ 02 - 7 THÀNH VIÊN BẮT BUỘC)</t>
         </is>
       </c>
-      <c r="C44" s="2" t="n"/>
-      <c r="D44" s="2" t="n"/>
-      <c r="E44" s="2" t="n"/>
-      <c r="F44" s="2" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>D01</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Chủ tịch HĐ Đề cương (Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>Nguyễn Công Khẩn</t>
-        </is>
-      </c>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>GS.TS.</t>
-        </is>
-      </c>
-      <c r="E45" s="3" t="inlineStr">
-        <is>
-          <t>Hội đồng Đạo đức Y sinh Quốc gia</t>
-        </is>
-      </c>
-      <c r="F45">
-        <f>IF(ISBLANK(C45), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
-        <v/>
-      </c>
+      <c r="C45" s="2" t="n"/>
+      <c r="D45" s="2" t="n"/>
+      <c r="E45" s="2" t="n"/>
+      <c r="F45" s="2" t="n"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>D02</t>
+          <t>D01</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 1 (Bắt buộc)</t>
+          <t>Chủ tịch HĐ Đề cương (Bắt buộc)</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Xuân Ninh</t>
+          <t>Nguyễn Công Khẩn</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>PGS.TS.BS.</t>
+          <t>GS.TS.</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Viện Y học Ứng dụng Việt Nam</t>
+          <t>Hội đồng Đạo đức Y sinh Quốc gia</t>
         </is>
       </c>
       <c r="F46">
@@ -1472,27 +1460,27 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>D03</t>
+          <t>D02</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 2 (Bắt buộc)</t>
+          <t>Ủy viên Phản biện 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Trần Quang Trung</t>
+          <t>Nguyễn Xuân Ninh</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>PGS.TS.</t>
+          <t>PGS.TS.BS.</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Hiệp hội Sữa Việt Nam</t>
+          <t>Viện Y học Ứng dụng Việt Nam</t>
         </is>
       </c>
       <c r="F47">
@@ -1503,27 +1491,27 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>D04</t>
+          <t>D03</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đề cương 1 (Bắt buộc)</t>
+          <t>Ủy viên Phản biện 2 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Lê Bạch Mai</t>
+          <t>Trần Quang Trung</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>PGS.TS.BS.</t>
+          <t>PGS.TS.</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Nguyên Phó Viện trưởng Viện Dinh dưỡng QG</t>
+          <t>Hiệp hội Sữa Việt Nam</t>
         </is>
       </c>
       <c r="F48">
@@ -1534,17 +1522,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>D05</t>
+          <t>D04</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đề cương 2 (Bắt buộc)</t>
+          <t>Ủy viên HĐ Đề cương 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Thị Lâm</t>
+          <t>Lê Bạch Mai</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -1565,28 +1553,43 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>D06</t>
+          <t>D05</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 3 (Tùy chọn)</t>
+          <t>Ủy viên HĐ Đề cương 2 (Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Nguyễn Thị Lâm</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>PGS.TS.BS.</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>Nguyên Phó Viện trưởng Viện Dinh dưỡng QG</t>
         </is>
       </c>
       <c r="F50">
-        <f>IF(ISBLANK(C50), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C50), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>D07</t>
+          <t>D06</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đề cương 3 (Tùy chọn)</t>
+          <t>Ủy viên Phản biện 3 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F51">
@@ -1597,12 +1600,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>D08</t>
+          <t>D07</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đề cương 4 (Tùy chọn)</t>
+          <t>Ủy viên HĐ Đề cương 3 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F52">
@@ -1613,48 +1616,33 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>D09</t>
+          <t>D08</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Thư ký HĐ Đề cương 1 (Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C53" s="3" t="inlineStr">
-        <is>
-          <t>Hoàng Hà Linh</t>
-        </is>
-      </c>
-      <c r="D53" s="3" t="inlineStr">
-        <is>
-          <t>Thạc sĩ</t>
-        </is>
-      </c>
-      <c r="E53" s="3" t="inlineStr">
-        <is>
-          <t>Trung tâm NCKH - Viện VIAM</t>
+          <t>Ủy viên HĐ Đề cương 4 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F53">
-        <f>IF(ISBLANK(C53), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C53), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1">
       <c r="A54" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>D09</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Thư ký HĐ Đề cương 2 (Bắt buộc)</t>
+          <t>Thư ký HĐ Đề cương 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Trương Phan Hồng Hà</t>
+          <t>Hoàng Hà Linh</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -1664,7 +1652,7 @@
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>Viện Y học Ứng dụng Việt Nam</t>
+          <t>Trung tâm NCKH - Viện VIAM</t>
         </is>
       </c>
       <c r="F54">
@@ -1673,76 +1661,76 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Thư ký HĐ Đề cương 2 (Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Trương Phan Hồng Hà</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Thạc sĩ</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Viện Y học Ứng dụng Việt Nam</t>
+        </is>
+      </c>
+      <c r="F55">
+        <f>IF(ISBLANK(C55), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>SEC_E</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>PHẦN E: HỘI ĐỒNG ĐÁNH GIÁ NGHIỆM THU (HĐ 03 - 7 THÀNH VIÊN BẮT BUỘC)</t>
         </is>
       </c>
-      <c r="C55" s="2" t="n"/>
-      <c r="D55" s="2" t="n"/>
-      <c r="E55" s="2" t="n"/>
-      <c r="F55" s="2" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>E01</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Chủ tịch HĐ Nghiệm thu (Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C56" s="3" t="inlineStr">
-        <is>
-          <t>Phạm Văn Hoàn</t>
-        </is>
-      </c>
-      <c r="D56" s="3" t="inlineStr">
-        <is>
-          <t>PGS.TS.</t>
-        </is>
-      </c>
-      <c r="E56" s="3" t="inlineStr">
-        <is>
-          <t>Viện Y học Ứng dụng Việt Nam</t>
-        </is>
-      </c>
-      <c r="F56">
-        <f>IF(ISBLANK(C56), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
-        <v/>
-      </c>
+      <c r="C56" s="2" t="n"/>
+      <c r="D56" s="2" t="n"/>
+      <c r="E56" s="2" t="n"/>
+      <c r="F56" s="2" t="n"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>E02</t>
+          <t>E01</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 1 (Bắt buộc)</t>
+          <t>Chủ tịch HĐ Nghiệm thu (Bắt buộc)</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Công Khẩn</t>
+          <t>Phạm Văn Hoàn</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>GS.TS.</t>
+          <t>PGS.TS.</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>Hội đồng Đạo đức Y sinh Quốc gia</t>
+          <t>Viện Y học Ứng dụng Việt Nam</t>
         </is>
       </c>
       <c r="F57">
@@ -1753,27 +1741,27 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>E03</t>
+          <t>E02</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 2 (Bắt buộc)</t>
+          <t>Ủy viên Phản biện 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Thị Lâm</t>
+          <t>Nguyễn Công Khẩn</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>PGS.TS.BS.</t>
+          <t>GS.TS.</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>Nguyên Phó Viện trưởng Viện Dinh dưỡng QG</t>
+          <t>Hội đồng Đạo đức Y sinh Quốc gia</t>
         </is>
       </c>
       <c r="F58">
@@ -1784,27 +1772,27 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>E04</t>
+          <t>E03</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Nghiệm thu 1 (Bắt buộc)</t>
+          <t>Ủy viên Phản biện 2 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Ninh Thị Nhung</t>
+          <t>Nguyễn Thị Lâm</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>PGS.TS.</t>
+          <t>PGS.TS.BS.</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>Trường Đại học Y Dược Thái Bình</t>
+          <t>Nguyên Phó Viện trưởng Viện Dinh dưỡng QG</t>
         </is>
       </c>
       <c r="F59">
@@ -1815,17 +1803,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>E05</t>
+          <t>E04</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Nghiệm thu 2 (Bắt buộc)</t>
+          <t>Ủy viên HĐ Nghiệm thu 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>Trần Văn Ơn</t>
+          <t>Ninh Thị Nhung</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
@@ -1835,7 +1823,7 @@
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>Trường Đại học Dược Hà Nội</t>
+          <t>Trường Đại học Y Dược Thái Bình</t>
         </is>
       </c>
       <c r="F60">
@@ -1846,28 +1834,43 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>E06</t>
+          <t>E05</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 3 (Tùy chọn)</t>
+          <t>Ủy viên HĐ Nghiệm thu 2 (Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>Trần Văn Ơn</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>PGS.TS.</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>Trường Đại học Dược Hà Nội</t>
         </is>
       </c>
       <c r="F61">
-        <f>IF(ISBLANK(C61), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C61), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>E07</t>
+          <t>E06</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Nghiệm thu 3 (Tùy chọn)</t>
+          <t>Ủy viên Phản biện 3 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F62">
@@ -1878,12 +1881,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>E08</t>
+          <t>E07</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Nghiệm thu 4 (Tùy chọn)</t>
+          <t>Ủy viên HĐ Nghiệm thu 3 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F63">
@@ -1894,53 +1897,38 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>E09</t>
+          <t>E08</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Thư ký HĐ Nghiệm thu 1 (Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C64" s="3" t="inlineStr">
-        <is>
-          <t>Hoàng Hà Linh</t>
-        </is>
-      </c>
-      <c r="D64" s="3" t="inlineStr">
-        <is>
-          <t>PGS.TS.BS.</t>
-        </is>
-      </c>
-      <c r="E64" s="3" t="inlineStr">
-        <is>
-          <t>Viện Y học Ứng dụng Việt Nam</t>
+          <t>Ủy viên HĐ Nghiệm thu 4 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F64">
-        <f>IF(ISBLANK(C64), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C64), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1">
       <c r="A65" t="inlineStr">
         <is>
-          <t>E10</t>
+          <t>E09</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Thư ký HĐ Nghiệm thu 2 (Bắt buộc)</t>
+          <t>Thư ký HĐ Nghiệm thu 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Trương Phan Hồng Hà</t>
+          <t>Hoàng Hà Linh</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Thạc sĩ</t>
+          <t>PGS.TS.BS.</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
@@ -1954,92 +1942,92 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="inlineStr">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Thư ký HĐ Nghiệm thu 2 (Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>Trương Phan Hồng Hà</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>Thạc sĩ</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>Viện Y học Ứng dụng Việt Nam</t>
+        </is>
+      </c>
+      <c r="F66">
+        <f>IF(ISBLANK(C66), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
         <is>
           <t>SEC_F</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="B67" s="2" t="inlineStr">
         <is>
           <t>PHẦN F: LÝ LỊCH KHOA HỌC CHUYÊN GIA (CV CHỦ NHIỆM BẮT BUỘC &amp; CV THÀNH VIÊN TÙY CHỌN)</t>
         </is>
       </c>
-      <c r="C66" s="2" t="n"/>
-      <c r="D66" s="2" t="n"/>
-      <c r="E66" s="2" t="n"/>
-      <c r="F66" s="2" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>F01</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>Hồ sơ Chủ nhiệm đề tài (Bắt buộc - File mặc định cho HĐ Đạo đức)</t>
-        </is>
-      </c>
-      <c r="C67" s="3" t="inlineStr">
-        <is>
-          <t>Trương Hồng Sơn</t>
-        </is>
-      </c>
-      <c r="D67" s="3" t="inlineStr">
-        <is>
-          <t>Chủ nhiệm đề tài</t>
-        </is>
-      </c>
-      <c r="E67" s="3" t="inlineStr">
-        <is>
-          <t>Lý lịch khoa học - Trương Hồng Sơn.docx</t>
-        </is>
-      </c>
-      <c r="F67">
-        <f>IF(ISBLANK(C67), "❌ CHƯA ĐIỀN THÔNG TIN CNĐT (BÁO LỖI)", IF(OR(ISBLANK(D67), ISBLANK(E67)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV Mặc định Đạo đức"))</f>
-        <v/>
-      </c>
+      <c r="C67" s="2" t="n"/>
+      <c r="D67" s="2" t="n"/>
+      <c r="E67" s="2" t="n"/>
+      <c r="F67" s="2" t="n"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>F02</t>
+          <t>F01</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Hồ sơ Đồng Chủ nhiệm (Tùy chọn)</t>
+          <t>Hồ sơ Chủ nhiệm đề tài (Bắt buộc - File mặc định cho HĐ Đạo đức)</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>Trương Hồng Sơn</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>Chủ nhiệm đề tài</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>Lý lịch khoa học - Trương Hồng Sơn.docx</t>
         </is>
       </c>
       <c r="F68">
-        <f>IF(ISBLANK(C68), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D68), ISBLANK(E68)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
+        <f>IF(ISBLANK(C68), "❌ CHƯA ĐIỀN THÔNG TIN CNĐT (BÁO LỖI)", IF(OR(ISBLANK(D68), ISBLANK(E68)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV Mặc định Đạo đức"))</f>
         <v/>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>F03</t>
+          <t>F02</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Hồ sơ Thư ký Đề tài (Tùy chọn)</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>Lưu Liên Hương</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>Thư ký Đề tài</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>Lý lịch khoa học_Liên Hương-2023.docx</t>
+          <t>Hồ sơ Đồng Chủ nhiệm (Tùy chọn)</t>
         </is>
       </c>
       <c r="F69">
@@ -2050,12 +2038,27 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>F04</t>
+          <t>F03</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 4 (Tùy chọn)</t>
+          <t>Hồ sơ Thư ký Đề tài (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Lưu Liên Hương</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Thư ký Đề tài</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Lý lịch khoa học_Liên Hương-2023.docx</t>
         </is>
       </c>
       <c r="F70">
@@ -2066,12 +2069,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>F05</t>
+          <t>F04</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 5 (Tùy chọn)</t>
+          <t>Hồ sơ Chuyên gia / Thành viên 4 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F71">
@@ -2082,12 +2085,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>F06</t>
+          <t>F05</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 6 (Tùy chọn)</t>
+          <t>Hồ sơ Chuyên gia / Thành viên 5 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F72">
@@ -2098,12 +2101,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>F07</t>
+          <t>F06</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 7 (Tùy chọn)</t>
+          <t>Hồ sơ Chuyên gia / Thành viên 6 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F73">
@@ -2114,12 +2117,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>F08</t>
+          <t>F07</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 8 (Tùy chọn)</t>
+          <t>Hồ sơ Chuyên gia / Thành viên 7 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F74">
@@ -2130,12 +2133,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>F09</t>
+          <t>F08</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 9 (Tùy chọn)</t>
+          <t>Hồ sơ Chuyên gia / Thành viên 8 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F75">
@@ -2146,16 +2149,32 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>F10</t>
+          <t>F09</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 10 (Tùy chọn)</t>
+          <t>Hồ sơ Chuyên gia / Thành viên 9 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F76">
         <f>IF(ISBLANK(C76), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D76), ISBLANK(E76)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>F10</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Hồ sơ Chuyên gia / Thành viên 10 (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="F77">
+        <f>IF(ISBLANK(C77), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D77), ISBLANK(E77)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
         <v/>
       </c>
     </row>
@@ -2174,7 +2193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F76"/>
+  <dimension ref="A1:F77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="8.5" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2361,65 +2380,68 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>A07</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Địa điểm triển khai nghiên cứu (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n"/>
+      <c r="D12" s="3" t="n"/>
+      <c r="E12" s="3" t="n"/>
+      <c r="F12">
+        <f>IF(ISBLANK(C12), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>SEC_B</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>PHẦN B: BAN CHỦ NHIỆM &amp; NGHIÊN CỨU VIÊN ĐỀ TÀI (TỐI ĐA 20 NGƯỜI)</t>
         </is>
       </c>
-      <c r="C12" s="2" t="n"/>
-      <c r="D12" s="2" t="n"/>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>B01</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Chủ nhiệm đề tài (CNĐT - Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="n"/>
-      <c r="D13" s="3" t="n"/>
-      <c r="E13" s="3" t="n"/>
-      <c r="F13">
-        <f>IF(ISBLANK(C13), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
-        <v/>
-      </c>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>B02</t>
+          <t>B01</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Đồng Chủ nhiệm đề tài (Tùy chọn)</t>
-        </is>
-      </c>
+          <t>Chủ nhiệm đề tài (CNĐT - Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n"/>
+      <c r="D14" s="3" t="n"/>
+      <c r="E14" s="3" t="n"/>
       <c r="F14">
-        <f>IF(ISBLANK(C14), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C14), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>B03</t>
+          <t>B02</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Thư ký Đề tài (Khác Thư ký HĐ - Tùy chọn)</t>
+          <t>Đồng Chủ nhiệm đề tài (Tùy chọn)</t>
         </is>
       </c>
       <c r="F15">
@@ -2430,12 +2452,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>B04</t>
+          <t>B03</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 1</t>
+          <t>Thư ký Đề tài (Khác Thư ký HĐ - Tùy chọn)</t>
         </is>
       </c>
       <c r="F16">
@@ -2446,12 +2468,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>B05</t>
+          <t>B04</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 2</t>
+          <t>Nghiên cứu viên 1</t>
         </is>
       </c>
       <c r="F17">
@@ -2462,12 +2484,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>B06</t>
+          <t>B05</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 3</t>
+          <t>Nghiên cứu viên 2</t>
         </is>
       </c>
       <c r="F18">
@@ -2478,12 +2500,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>B07</t>
+          <t>B06</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 4</t>
+          <t>Nghiên cứu viên 3</t>
         </is>
       </c>
       <c r="F19">
@@ -2494,12 +2516,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>B08</t>
+          <t>B07</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 5</t>
+          <t>Nghiên cứu viên 4</t>
         </is>
       </c>
       <c r="F20">
@@ -2510,12 +2532,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>B09</t>
+          <t>B08</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 6</t>
+          <t>Nghiên cứu viên 5</t>
         </is>
       </c>
       <c r="F21">
@@ -2526,12 +2548,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>B10</t>
+          <t>B09</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 7</t>
+          <t>Nghiên cứu viên 6</t>
         </is>
       </c>
       <c r="F22">
@@ -2542,12 +2564,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>B11</t>
+          <t>B10</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 8</t>
+          <t>Nghiên cứu viên 7</t>
         </is>
       </c>
       <c r="F23">
@@ -2558,12 +2580,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>B12</t>
+          <t>B11</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 9</t>
+          <t>Nghiên cứu viên 8</t>
         </is>
       </c>
       <c r="F24">
@@ -2574,12 +2596,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>B13</t>
+          <t>B12</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 10</t>
+          <t>Nghiên cứu viên 9</t>
         </is>
       </c>
       <c r="F25">
@@ -2590,12 +2612,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>B14</t>
+          <t>B13</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 11</t>
+          <t>Nghiên cứu viên 10</t>
         </is>
       </c>
       <c r="F26">
@@ -2606,12 +2628,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>B15</t>
+          <t>B14</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 12</t>
+          <t>Nghiên cứu viên 11</t>
         </is>
       </c>
       <c r="F27">
@@ -2622,12 +2644,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>B16</t>
+          <t>B15</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 13</t>
+          <t>Nghiên cứu viên 12</t>
         </is>
       </c>
       <c r="F28">
@@ -2638,12 +2660,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>B17</t>
+          <t>B16</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 14</t>
+          <t>Nghiên cứu viên 13</t>
         </is>
       </c>
       <c r="F29">
@@ -2654,12 +2676,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>B18</t>
+          <t>B17</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 15</t>
+          <t>Nghiên cứu viên 14</t>
         </is>
       </c>
       <c r="F30">
@@ -2670,17 +2692,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>B19</t>
+          <t>B18</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 16</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>(Để trống tên theo quy định)</t>
+          <t>Nghiên cứu viên 15</t>
         </is>
       </c>
       <c r="F31">
@@ -2691,12 +2708,12 @@
     <row r="32" ht="15" customHeight="1">
       <c r="A32" t="inlineStr">
         <is>
-          <t>B20</t>
+          <t>B19</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 17</t>
+          <t>Nghiên cứu viên 16</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2710,49 +2727,51 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>B20</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Nghiên cứu viên 17</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>(Để trống tên theo quy định)</t>
+        </is>
+      </c>
+      <c r="F33">
+        <f>IF(ISBLANK(C33), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>SEC_C</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>PHẦN C: HỘI ĐỒNG ĐẠO ĐỨC TRONG NGHIÊN CỨU (HĐ 01 - 7 THÀNH VIÊN BẮT BUỘC)</t>
         </is>
       </c>
-      <c r="C33" s="2" t="n"/>
-      <c r="D33" s="2" t="n"/>
-      <c r="E33" s="2" t="n"/>
-      <c r="F33" s="2" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>C01</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Chủ tịch HĐ Đạo đức (Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="n"/>
-      <c r="D34" s="3" t="n"/>
-      <c r="E34" s="3" t="n"/>
-      <c r="F34">
-        <f>IF(ISBLANK(C34), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
-        <v/>
-      </c>
+      <c r="C34" s="2" t="n"/>
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>C02</t>
+          <t>C01</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 1 (Bắt buộc)</t>
+          <t>Chủ tịch HĐ Đạo đức (Bắt buộc)</t>
         </is>
       </c>
       <c r="C35" s="3" t="n"/>
@@ -2766,12 +2785,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>C03</t>
+          <t>C02</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 2 (Bắt buộc)</t>
+          <t>Ủy viên Phản biện 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C36" s="3" t="n"/>
@@ -2785,12 +2804,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>C04</t>
+          <t>C03</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đạo đức 1 (Bắt buộc)</t>
+          <t>Ủy viên Phản biện 2 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C37" s="3" t="n"/>
@@ -2804,12 +2823,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>C05</t>
+          <t>C04</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đạo đức 2 (Bắt buộc)</t>
+          <t>Ủy viên HĐ Đạo đức 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C38" s="3" t="n"/>
@@ -2823,28 +2842,31 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>C06</t>
+          <t>C05</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 3 (Tùy chọn)</t>
-        </is>
-      </c>
+          <t>Ủy viên HĐ Đạo đức 2 (Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="n"/>
+      <c r="D39" s="3" t="n"/>
+      <c r="E39" s="3" t="n"/>
       <c r="F39">
-        <f>IF(ISBLANK(C39), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C39), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>C07</t>
+          <t>C06</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đạo đức 3 (Tùy chọn)</t>
+          <t>Ủy viên Phản biện 3 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F40">
@@ -2855,12 +2877,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>C08</t>
+          <t>C07</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đạo đức 4 (Tùy chọn)</t>
+          <t>Ủy viên HĐ Đạo đức 3 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F41">
@@ -2871,31 +2893,28 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>C09</t>
+          <t>C08</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Thư ký HĐ Đạo đức 1 (Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="n"/>
-      <c r="D42" s="3" t="n"/>
-      <c r="E42" s="3" t="n"/>
+          <t>Ủy viên HĐ Đạo đức 4 (Tùy chọn)</t>
+        </is>
+      </c>
       <c r="F42">
-        <f>IF(ISBLANK(C42), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C42), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" t="inlineStr">
         <is>
-          <t>C10</t>
+          <t>C09</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Thư ký HĐ Đạo đức 2 (Bắt buộc)</t>
+          <t>Thư ký HĐ Đạo đức 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C43" s="3" t="n"/>
@@ -2907,49 +2926,49 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Thư ký HĐ Đạo đức 2 (Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="n"/>
+      <c r="D44" s="3" t="n"/>
+      <c r="E44" s="3" t="n"/>
+      <c r="F44">
+        <f>IF(ISBLANK(C44), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>SEC_D</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>PHẦN D: HỘI ĐỒNG KHOA HỌC XÉT DUYỆT ĐỀ CƯƠNG (HĐ 02 - 7 THÀNH VIÊN BẮT BUỘC)</t>
         </is>
       </c>
-      <c r="C44" s="2" t="n"/>
-      <c r="D44" s="2" t="n"/>
-      <c r="E44" s="2" t="n"/>
-      <c r="F44" s="2" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>D01</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Chủ tịch HĐ Đề cương (Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="n"/>
-      <c r="D45" s="3" t="n"/>
-      <c r="E45" s="3" t="n"/>
-      <c r="F45">
-        <f>IF(ISBLANK(C45), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
-        <v/>
-      </c>
+      <c r="C45" s="2" t="n"/>
+      <c r="D45" s="2" t="n"/>
+      <c r="E45" s="2" t="n"/>
+      <c r="F45" s="2" t="n"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>D02</t>
+          <t>D01</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 1 (Bắt buộc)</t>
+          <t>Chủ tịch HĐ Đề cương (Bắt buộc)</t>
         </is>
       </c>
       <c r="C46" s="3" t="n"/>
@@ -2963,12 +2982,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>D03</t>
+          <t>D02</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 2 (Bắt buộc)</t>
+          <t>Ủy viên Phản biện 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C47" s="3" t="n"/>
@@ -2982,12 +3001,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>D04</t>
+          <t>D03</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đề cương 1 (Bắt buộc)</t>
+          <t>Ủy viên Phản biện 2 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C48" s="3" t="n"/>
@@ -3001,12 +3020,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>D05</t>
+          <t>D04</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đề cương 2 (Bắt buộc)</t>
+          <t>Ủy viên HĐ Đề cương 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C49" s="3" t="n"/>
@@ -3020,28 +3039,31 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>D06</t>
+          <t>D05</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 3 (Tùy chọn)</t>
-        </is>
-      </c>
+          <t>Ủy viên HĐ Đề cương 2 (Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="n"/>
+      <c r="D50" s="3" t="n"/>
+      <c r="E50" s="3" t="n"/>
       <c r="F50">
-        <f>IF(ISBLANK(C50), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C50), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>D07</t>
+          <t>D06</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đề cương 3 (Tùy chọn)</t>
+          <t>Ủy viên Phản biện 3 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F51">
@@ -3052,12 +3074,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>D08</t>
+          <t>D07</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đề cương 4 (Tùy chọn)</t>
+          <t>Ủy viên HĐ Đề cương 3 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F52">
@@ -3068,31 +3090,28 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>D09</t>
+          <t>D08</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Thư ký HĐ Đề cương 1 (Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C53" s="3" t="n"/>
-      <c r="D53" s="3" t="n"/>
-      <c r="E53" s="3" t="n"/>
+          <t>Ủy viên HĐ Đề cương 4 (Tùy chọn)</t>
+        </is>
+      </c>
       <c r="F53">
-        <f>IF(ISBLANK(C53), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C53), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1">
       <c r="A54" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>D09</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Thư ký HĐ Đề cương 2 (Bắt buộc)</t>
+          <t>Thư ký HĐ Đề cương 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C54" s="3" t="n"/>
@@ -3104,49 +3123,49 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Thư ký HĐ Đề cương 2 (Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="n"/>
+      <c r="D55" s="3" t="n"/>
+      <c r="E55" s="3" t="n"/>
+      <c r="F55">
+        <f>IF(ISBLANK(C55), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>SEC_E</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>PHẦN E: HỘI ĐỒNG ĐÁNH GIÁ NGHIỆM THU (HĐ 03 - 7 THÀNH VIÊN BẮT BUỘC)</t>
         </is>
       </c>
-      <c r="C55" s="2" t="n"/>
-      <c r="D55" s="2" t="n"/>
-      <c r="E55" s="2" t="n"/>
-      <c r="F55" s="2" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>E01</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Chủ tịch HĐ Nghiệm thu (Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C56" s="3" t="n"/>
-      <c r="D56" s="3" t="n"/>
-      <c r="E56" s="3" t="n"/>
-      <c r="F56">
-        <f>IF(ISBLANK(C56), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
-        <v/>
-      </c>
+      <c r="C56" s="2" t="n"/>
+      <c r="D56" s="2" t="n"/>
+      <c r="E56" s="2" t="n"/>
+      <c r="F56" s="2" t="n"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>E02</t>
+          <t>E01</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 1 (Bắt buộc)</t>
+          <t>Chủ tịch HĐ Nghiệm thu (Bắt buộc)</t>
         </is>
       </c>
       <c r="C57" s="3" t="n"/>
@@ -3160,12 +3179,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>E03</t>
+          <t>E02</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 2 (Bắt buộc)</t>
+          <t>Ủy viên Phản biện 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C58" s="3" t="n"/>
@@ -3179,12 +3198,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>E04</t>
+          <t>E03</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Nghiệm thu 1 (Bắt buộc)</t>
+          <t>Ủy viên Phản biện 2 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C59" s="3" t="n"/>
@@ -3198,12 +3217,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>E05</t>
+          <t>E04</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Nghiệm thu 2 (Bắt buộc)</t>
+          <t>Ủy viên HĐ Nghiệm thu 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C60" s="3" t="n"/>
@@ -3217,28 +3236,31 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>E06</t>
+          <t>E05</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 3 (Tùy chọn)</t>
-        </is>
-      </c>
+          <t>Ủy viên HĐ Nghiệm thu 2 (Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="n"/>
+      <c r="D61" s="3" t="n"/>
+      <c r="E61" s="3" t="n"/>
       <c r="F61">
-        <f>IF(ISBLANK(C61), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C61), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>E07</t>
+          <t>E06</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Nghiệm thu 3 (Tùy chọn)</t>
+          <t>Ủy viên Phản biện 3 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F62">
@@ -3249,12 +3271,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>E08</t>
+          <t>E07</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Nghiệm thu 4 (Tùy chọn)</t>
+          <t>Ủy viên HĐ Nghiệm thu 3 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F63">
@@ -3265,31 +3287,28 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>E09</t>
+          <t>E08</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Thư ký HĐ Nghiệm thu 1 (Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C64" s="3" t="n"/>
-      <c r="D64" s="3" t="n"/>
-      <c r="E64" s="3" t="n"/>
+          <t>Ủy viên HĐ Nghiệm thu 4 (Tùy chọn)</t>
+        </is>
+      </c>
       <c r="F64">
-        <f>IF(ISBLANK(C64), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C64), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1">
       <c r="A65" t="inlineStr">
         <is>
-          <t>E10</t>
+          <t>E09</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Thư ký HĐ Nghiệm thu 2 (Bắt buộc)</t>
+          <t>Thư ký HĐ Nghiệm thu 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C65" s="3" t="n"/>
@@ -3301,65 +3320,68 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="inlineStr">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Thư ký HĐ Nghiệm thu 2 (Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="n"/>
+      <c r="D66" s="3" t="n"/>
+      <c r="E66" s="3" t="n"/>
+      <c r="F66">
+        <f>IF(ISBLANK(C66), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
         <is>
           <t>SEC_F</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="B67" s="2" t="inlineStr">
         <is>
           <t>PHẦN F: LÝ LỊCH KHOA HỌC CHUYÊN GIA (CV CHỦ NHIỆM BẮT BUỘC &amp; CV THÀNH VIÊN TÙY CHỌN)</t>
         </is>
       </c>
-      <c r="C66" s="2" t="n"/>
-      <c r="D66" s="2" t="n"/>
-      <c r="E66" s="2" t="n"/>
-      <c r="F66" s="2" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>F01</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>Hồ sơ Chủ nhiệm đề tài (Bắt buộc - File mặc định cho HĐ Đạo đức)</t>
-        </is>
-      </c>
-      <c r="C67" s="3" t="n"/>
-      <c r="D67" s="3" t="n"/>
-      <c r="E67" s="3" t="n"/>
-      <c r="F67">
-        <f>IF(ISBLANK(C67), "❌ CHƯA ĐIỀN THÔNG TIN CNĐT (BÁO LỖI)", IF(OR(ISBLANK(D67), ISBLANK(E67)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV Mặc định Đạo đức"))</f>
-        <v/>
-      </c>
+      <c r="C67" s="2" t="n"/>
+      <c r="D67" s="2" t="n"/>
+      <c r="E67" s="2" t="n"/>
+      <c r="F67" s="2" t="n"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>F02</t>
+          <t>F01</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Hồ sơ Đồng Chủ nhiệm (Tùy chọn)</t>
-        </is>
-      </c>
+          <t>Hồ sơ Chủ nhiệm đề tài (Bắt buộc - File mặc định cho HĐ Đạo đức)</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="n"/>
+      <c r="D68" s="3" t="n"/>
+      <c r="E68" s="3" t="n"/>
       <c r="F68">
-        <f>IF(ISBLANK(C68), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D68), ISBLANK(E68)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
+        <f>IF(ISBLANK(C68), "❌ CHƯA ĐIỀN THÔNG TIN CNĐT (BÁO LỖI)", IF(OR(ISBLANK(D68), ISBLANK(E68)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV Mặc định Đạo đức"))</f>
         <v/>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>F03</t>
+          <t>F02</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Hồ sơ Thư ký Đề tài (Tùy chọn)</t>
+          <t>Hồ sơ Đồng Chủ nhiệm (Tùy chọn)</t>
         </is>
       </c>
       <c r="F69">
@@ -3370,12 +3392,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>F04</t>
+          <t>F03</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 4 (Tùy chọn)</t>
+          <t>Hồ sơ Thư ký Đề tài (Tùy chọn)</t>
         </is>
       </c>
       <c r="F70">
@@ -3386,12 +3408,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>F05</t>
+          <t>F04</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 5 (Tùy chọn)</t>
+          <t>Hồ sơ Chuyên gia / Thành viên 4 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F71">
@@ -3402,12 +3424,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>F06</t>
+          <t>F05</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 6 (Tùy chọn)</t>
+          <t>Hồ sơ Chuyên gia / Thành viên 5 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F72">
@@ -3418,12 +3440,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>F07</t>
+          <t>F06</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 7 (Tùy chọn)</t>
+          <t>Hồ sơ Chuyên gia / Thành viên 6 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F73">
@@ -3434,12 +3456,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>F08</t>
+          <t>F07</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 8 (Tùy chọn)</t>
+          <t>Hồ sơ Chuyên gia / Thành viên 7 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F74">
@@ -3450,12 +3472,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>F09</t>
+          <t>F08</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 9 (Tùy chọn)</t>
+          <t>Hồ sơ Chuyên gia / Thành viên 8 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F75">
@@ -3466,16 +3488,32 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>F10</t>
+          <t>F09</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 10 (Tùy chọn)</t>
+          <t>Hồ sơ Chuyên gia / Thành viên 9 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F76">
         <f>IF(ISBLANK(C76), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D76), ISBLANK(E76)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>F10</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Hồ sơ Chuyên gia / Thành viên 10 (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="F77">
+        <f>IF(ISBLANK(C77), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D77), ISBLANK(E77)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: relocate expert CV PDFs into CV chuyên gia/, drop redundant .doc masters, populate sample checklist F04-F08
Also removes Task 5's temporary skip on
test_real_checklist_expert_cvs_has_at_least_one_entry now that F04-F08
carry real data, and re-bases
test_convert_doc_templates::test_convert_one_preserves_table_count onto
a .doc fixture it generates itself via SaveAs2(FileFormat=WD_FORMAT_DOC)
from the surviving .docx template, since its original .doc fixture was
one of the 7 files deleted here.
</commit_message>
<xml_diff>
--- a/Form checklist hồ sơ dự án.xlsx
+++ b/Form checklist hồ sơ dự án.xlsx
@@ -2077,6 +2077,21 @@
           <t>Hồ sơ Chuyên gia / Thành viên 4 (Tùy chọn)</t>
         </is>
       </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Nguyễn Công Khẩn</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Chuyên gia hội đồng</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>TM-Gs. Nguyen Cong Khan.pdf</t>
+        </is>
+      </c>
       <c r="F71">
         <f>IF(ISBLANK(C71), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D71), ISBLANK(E71)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
         <v/>
@@ -2093,6 +2108,21 @@
           <t>Hồ sơ Chuyên gia / Thành viên 5 (Tùy chọn)</t>
         </is>
       </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Hoàng Thị Thanh</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Chuyên gia hội đồng</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>TM-PGs. Hoang Thi Thanh.pdf</t>
+        </is>
+      </c>
       <c r="F72">
         <f>IF(ISBLANK(C72), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D72), ISBLANK(E72)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
         <v/>
@@ -2109,6 +2139,21 @@
           <t>Hồ sơ Chuyên gia / Thành viên 6 (Tùy chọn)</t>
         </is>
       </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Nguyễn Quang Dũng</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Chuyên gia hội đồng</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>TM-PGs. Nguyen Quang Dung.pdf</t>
+        </is>
+      </c>
       <c r="F73">
         <f>IF(ISBLANK(C73), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D73), ISBLANK(E73)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
         <v/>
@@ -2125,6 +2170,21 @@
           <t>Hồ sơ Chuyên gia / Thành viên 7 (Tùy chọn)</t>
         </is>
       </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Trần Quang Trung</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Chuyên gia hội đồng</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>TM-PGs. Tran Quang Trung.pdf</t>
+        </is>
+      </c>
       <c r="F74">
         <f>IF(ISBLANK(C74), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D74), ISBLANK(E74)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
         <v/>
@@ -2139,6 +2199,21 @@
       <c r="B75" t="inlineStr">
         <is>
           <t>Hồ sơ Chuyên gia / Thành viên 8 (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Nguyễn Hùng Long</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Chuyên gia hội đồng</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>TM-Ts. Nguyen Hung Long.pdf</t>
         </is>
       </c>
       <c r="F75">

</xml_diff>

<commit_message>
fix: clear dangling F03 CV filename reference in real checklist
F03 (Lưu Liên Hương, Thư ký Đề tài) pointed to
"Lý lịch khoa học_Liên Hương-2023.docx", a file that does not exist in
CV chuyên gia/. This is pre-existing user data that predates Task 6 and
was invisible before read_expert_cvs (Task 5) started reading F02-F10.
Left in place it would make copy_expert_cvs() (Task 7) raise
FileNotFoundError against the real checklist.

Per user decision, clear only the filename cell (column 5) and keep the
name and role so the user can re-enter the filename once the file
exists. read_expert_cvs now returns exactly the 5 F04-F08 entries this
task populated.
</commit_message>
<xml_diff>
--- a/Form checklist hồ sơ dự án.xlsx
+++ b/Form checklist hồ sơ dự án.xlsx
@@ -2056,11 +2056,6 @@
           <t>Thư ký Đề tài</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>Lý lịch khoa học_Liên Hương-2023.docx</t>
-        </is>
-      </c>
       <c r="F70">
         <f>IF(ISBLANK(C70), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D70), ISBLANK(E70)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
         <v/>

</xml_diff>

<commit_message>
feat: add CV filename and research-type Excel dropdowns via a manually-run refresh script
</commit_message>
<xml_diff>
--- a/Form checklist hồ sơ dự án.xlsx
+++ b/Form checklist hồ sơ dự án.xlsx
@@ -8,6 +8,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đề tài - Bánh ăn dặm VIAM 2027" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đề tài - Mẫu trắng dự án mới" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Lists" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -3592,6 +3593,70 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="E68 E69 E70 E71 E72 E73 E74 E75 E76 E77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>='_Lists'!$A$1:$A$6</formula1>
+    </dataValidation>
+    <dataValidation sqref="C7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"TVCT_ĐGHQ,TNLS"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Lý lịch khoa học - Trương Hồng Sơn.docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TM-Gs. Nguyen Cong Khan.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TM-PGs. Hoang Thi Thanh.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TM-PGs. Nguyen Quang Dung.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TM-PGs. Tran Quang Trung.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TM-Ts. Nguyen Hung Long.pdf</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add _Tokens sheet migration with 12 default token definitions
</commit_message>
<xml_diff>
--- a/Form checklist hồ sơ dự án.xlsx
+++ b/Form checklist hồ sơ dự án.xlsx
@@ -9,6 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đề tài - Bánh ăn dặm VIAM 2027" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đề tài - Mẫu trắng dự án mới" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Lists" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Tokens" sheetId="4" state="hidden" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -3659,4 +3660,325 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>token_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>param</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TEN_DE_TAI</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>A01</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Tên đề tài</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NAM</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>A03</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Năm thực hiện hồ sơ</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DON_VI_CHU_TRI</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>A04</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Cơ quan chủ trì</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DON_VI_DOI_TAC</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>A06</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Cơ quan phối hợp</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CHU_NHIEM_HO_TEN</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>B01</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>person_ho_ten</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Chủ nhiệm đề tài - có học hàm/học vị</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CHU_NHIEM_TEN</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>B01</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>person_ten</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Chủ nhiệm đề tài - chỉ tên</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>DONG_CHU_NHIEM_TEN</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>B02</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>person_ten</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Đồng chủ nhiệm đề tài - chỉ tên</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DONG_CHU_NHIEM_HO_TEN</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>B02</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>person_ho_ten</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Đồng chủ nhiệm đề tài - có học hàm/học vị</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>THU_KY_DE_TAI</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>B03</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>person_ho_ten</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Thư ký đề tài</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>THOI_GIAN_BAT_DAU</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>A05</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>timeline_start</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Mốc bắt đầu (MM/YYYY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>THOI_GIAN_KET_THUC</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>A05</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>timeline_end</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Mốc kết thúc (MM/YYYY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>DIA_DIEM_TRIEN_KHAI</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>A07</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>raw_or_placeholder</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>……………………………</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Địa điểm triển khai nghiên cứu</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add _NhanSu shared person registry, seeded from existing project sheets
</commit_message>
<xml_diff>
--- a/Form checklist hồ sơ dự án.xlsx
+++ b/Form checklist hồ sơ dự án.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đề tài - Mẫu trắng dự án mới" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Lists" sheetId="3" state="hidden" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Tokens" sheetId="4" state="hidden" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_NhanSu" sheetId="5" state="hidden" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -3714,7 +3715,6 @@
           <t>raw</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>Tên đề tài</t>
@@ -3737,7 +3737,6 @@
           <t>raw</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>Năm thực hiện hồ sơ</t>
@@ -3760,7 +3759,6 @@
           <t>raw</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>Cơ quan chủ trì</t>
@@ -3783,7 +3781,6 @@
           <t>raw</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>Cơ quan phối hợp</t>
@@ -3806,7 +3803,6 @@
           <t>person_ho_ten</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>Chủ nhiệm đề tài - có học hàm/học vị</t>
@@ -3829,7 +3825,6 @@
           <t>person_ten</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>Chủ nhiệm đề tài - chỉ tên</t>
@@ -3852,7 +3847,6 @@
           <t>person_ten</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>Đồng chủ nhiệm đề tài - chỉ tên</t>
@@ -3875,7 +3869,6 @@
           <t>person_ho_ten</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>Đồng chủ nhiệm đề tài - có học hàm/học vị</t>
@@ -3898,7 +3891,6 @@
           <t>person_ho_ten</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>Thư ký đề tài</t>
@@ -3921,7 +3913,6 @@
           <t>timeline_start</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>Mốc bắt đầu (MM/YYYY)</t>
@@ -3944,7 +3935,6 @@
           <t>timeline_end</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>Mốc kết thúc (MM/YYYY)</t>
@@ -3975,6 +3965,327 @@
       <c r="E13" t="inlineStr">
         <is>
           <t>Địa điểm triển khai nghiên cứu</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ten</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>hoc_ham_hoc_vi</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>don_vi</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>dia_chi</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>sdt</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>cccd</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>mst</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>so_tk</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>ngan_hang</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Trương Hồng Sơn</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TS.BS.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Viện trưởng - Viện Y học Ứng dụng VN</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Lưu Liên Hương</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Thạc sĩ</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Trung tâm NCKH - Viện VIAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Lê Việt Anh</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Thạc sĩ</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Trung tâm NCKH - Viện VIAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Lê Minh Khánh</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Bác sĩ</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Phòng khám VIAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Nguyễn Công Khẩn</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>GS.TS.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Hội đồng Đạo đức Y sinh Quốc gia</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Nguyễn Xuân Ninh</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PGS.TS.BS.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Viện Y học Ứng dụng Việt Nam</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Lê Bạch Mai</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>PGS.TS.BS.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Nguyên Phó Viện trưởng Viện Dinh dưỡng QG</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Nguyễn Thị Lâm</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>PGS.TS.BS.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Nguyên Phó Viện trưởng Viện Dinh dưỡng QG</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Nguyễn Quang Dũng</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>PGS.TS.BS.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Bộ môn Dinh dưỡng - ĐH Y Hà Nội</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Hoàng Hà Linh</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Thạc sĩ</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Trung tâm NCKH - Viện VIAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Trương Phan Hồng Hà</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Thạc sĩ</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Viện Y học Ứng dụng Việt Nam</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Trần Quang Trung</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>PGS.TS.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Hiệp hội Sữa Việt Nam</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Phạm Văn Hoàn</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PGS.TS.</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Viện Y học Ứng dụng Việt Nam</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Ninh Thị Nhung</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>PGS.TS.</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Trường Đại học Y Dược Thái Bình</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Trần Văn Ơn</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>PGS.TS.</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Trường Đại học Dược Hà Nội</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: clear F03's undeclared CV name in the live VIAM 2027 checklist
</commit_message>
<xml_diff>
--- a/Form checklist hồ sơ dự án.xlsx
+++ b/Form checklist hồ sơ dự án.xlsx
@@ -2049,16 +2049,6 @@
           <t>Hồ sơ Thư ký Đề tài (Tùy chọn)</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>Lưu Liên Hương</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>Thư ký Đề tài</t>
-        </is>
-      </c>
       <c r="F70">
         <f>IF(ISBLANK(C70), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D70), ISBLANK(E70)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
         <v/>

</xml_diff>

<commit_message>
feat: add A08 'Đầu mối liên hệ' checklist field and its common token
</commit_message>
<xml_diff>
--- a/Form checklist hồ sơ dự án.xlsx
+++ b/Form checklist hồ sơ dự án.xlsx
@@ -9,8 +9,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đề tài - Bánh ăn dặm VIAM 2027" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đề tài - Mẫu trắng dự án mới" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Lists" sheetId="3" state="hidden" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Tokens" sheetId="4" state="hidden" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_NhanSu" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_NhanSu" sheetId="4" state="hidden" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Tokens" sheetId="5" state="hidden" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F77"/>
+  <dimension ref="A1:F78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="8.5" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -737,92 +737,80 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>A08</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Đầu mối liên hệ (họ tên, đơn vị, email, điện thoại - Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n"/>
+      <c r="D13" s="3" t="n"/>
+      <c r="E13" s="3" t="n"/>
+      <c r="F13">
+        <f>IF(ISBLANK(C13), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>SEC_B</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>PHẦN B: BAN CHỦ NHIỆM &amp; NGHIÊN CỨU VIÊN ĐỀ TÀI (TỐI ĐA 20 NGƯỜI)</t>
         </is>
       </c>
-      <c r="C13" s="2" t="n"/>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>B01</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Chủ nhiệm đề tài (CNĐT - Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Trương Hồng Sơn</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>TS.BS.</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>Viện trưởng - Viện Y học Ứng dụng VN</t>
-        </is>
-      </c>
-      <c r="F14">
-        <f>IF(ISBLANK(C14), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
-        <v/>
-      </c>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>B02</t>
+          <t>B01</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Đồng Chủ nhiệm đề tài (Tùy chọn)</t>
+          <t>Chủ nhiệm đề tài (CNĐT - Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Trương Hồng Sơn</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>TS.BS.</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Viện trưởng - Viện Y học Ứng dụng VN</t>
         </is>
       </c>
       <c r="F15">
-        <f>IF(ISBLANK(C15), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C15), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>B03</t>
+          <t>B02</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Thư ký Đề tài (Khác Thư ký HĐ - Tùy chọn)</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Lưu Liên Hương</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Thạc sĩ</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Trung tâm NCKH - Viện VIAM</t>
+          <t>Đồng Chủ nhiệm đề tài (Tùy chọn)</t>
         </is>
       </c>
       <c r="F16">
@@ -833,17 +821,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>B04</t>
+          <t>B03</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 1</t>
+          <t>Thư ký Đề tài (Khác Thư ký HĐ - Tùy chọn)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Lê Việt Anh</t>
+          <t>Lưu Liên Hương</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -864,27 +852,27 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>B05</t>
+          <t>B04</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 2</t>
+          <t>Nghiên cứu viên 1</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Lê Minh Khánh</t>
+          <t>Lê Việt Anh</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Bác sĩ</t>
+          <t>Thạc sĩ</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Phòng khám VIAM</t>
+          <t>Trung tâm NCKH - Viện VIAM</t>
         </is>
       </c>
       <c r="F18">
@@ -895,12 +883,27 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>B06</t>
+          <t>B05</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 3</t>
+          <t>Nghiên cứu viên 2</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Lê Minh Khánh</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Bác sĩ</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Phòng khám VIAM</t>
         </is>
       </c>
       <c r="F19">
@@ -911,12 +914,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>B07</t>
+          <t>B06</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 4</t>
+          <t>Nghiên cứu viên 3</t>
         </is>
       </c>
       <c r="F20">
@@ -927,12 +930,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>B08</t>
+          <t>B07</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 5</t>
+          <t>Nghiên cứu viên 4</t>
         </is>
       </c>
       <c r="F21">
@@ -943,12 +946,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>B09</t>
+          <t>B08</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 6</t>
+          <t>Nghiên cứu viên 5</t>
         </is>
       </c>
       <c r="F22">
@@ -959,12 +962,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>B10</t>
+          <t>B09</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 7</t>
+          <t>Nghiên cứu viên 6</t>
         </is>
       </c>
       <c r="F23">
@@ -975,12 +978,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>B11</t>
+          <t>B10</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 8</t>
+          <t>Nghiên cứu viên 7</t>
         </is>
       </c>
       <c r="F24">
@@ -991,12 +994,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>B12</t>
+          <t>B11</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 9</t>
+          <t>Nghiên cứu viên 8</t>
         </is>
       </c>
       <c r="F25">
@@ -1007,12 +1010,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>B13</t>
+          <t>B12</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 10</t>
+          <t>Nghiên cứu viên 9</t>
         </is>
       </c>
       <c r="F26">
@@ -1023,12 +1026,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>B14</t>
+          <t>B13</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 11</t>
+          <t>Nghiên cứu viên 10</t>
         </is>
       </c>
       <c r="F27">
@@ -1039,12 +1042,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>B15</t>
+          <t>B14</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 12</t>
+          <t>Nghiên cứu viên 11</t>
         </is>
       </c>
       <c r="F28">
@@ -1055,12 +1058,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>B16</t>
+          <t>B15</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 13</t>
+          <t>Nghiên cứu viên 12</t>
         </is>
       </c>
       <c r="F29">
@@ -1071,12 +1074,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>B17</t>
+          <t>B16</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 14</t>
+          <t>Nghiên cứu viên 13</t>
         </is>
       </c>
       <c r="F30">
@@ -1087,12 +1090,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>B18</t>
+          <t>B17</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 15</t>
+          <t>Nghiên cứu viên 14</t>
         </is>
       </c>
       <c r="F31">
@@ -1103,12 +1106,12 @@
     <row r="32" ht="15" customHeight="1">
       <c r="A32" t="inlineStr">
         <is>
-          <t>B19</t>
+          <t>B18</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 16</t>
+          <t>Nghiên cứu viên 15</t>
         </is>
       </c>
       <c r="F32">
@@ -1119,12 +1122,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>B20</t>
+          <t>B19</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 17</t>
+          <t>Nghiên cứu viên 16</t>
         </is>
       </c>
       <c r="F33">
@@ -1133,76 +1136,61 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>B20</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Nghiên cứu viên 17</t>
+        </is>
+      </c>
+      <c r="F34">
+        <f>IF(ISBLANK(C34), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>SEC_C</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>PHẦN C: HỘI ĐỒNG ĐẠO ĐỨC TRONG NGHIÊN CỨU (HĐ 01 - 7 THÀNH VIÊN BẮT BUỘC)</t>
         </is>
       </c>
-      <c r="C34" s="2" t="n"/>
-      <c r="D34" s="2" t="n"/>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="2" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>C01</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Chủ tịch HĐ Đạo đức (Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>Nguyễn Công Khẩn</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>GS.TS.</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr">
-        <is>
-          <t>Hội đồng Đạo đức Y sinh Quốc gia</t>
-        </is>
-      </c>
-      <c r="F35">
-        <f>IF(ISBLANK(C35), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
-        <v/>
-      </c>
+      <c r="C35" s="2" t="n"/>
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>C02</t>
+          <t>C01</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 1 (Bắt buộc)</t>
+          <t>Chủ tịch HĐ Đạo đức (Bắt buộc)</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Xuân Ninh</t>
+          <t>Nguyễn Công Khẩn</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>PGS.TS.BS.</t>
+          <t>GS.TS.</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Viện Y học Ứng dụng Việt Nam</t>
+          <t>Hội đồng Đạo đức Y sinh Quốc gia</t>
         </is>
       </c>
       <c r="F36">
@@ -1213,17 +1201,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>C03</t>
+          <t>C02</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 2 (Bắt buộc)</t>
+          <t>Ủy viên Phản biện 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Lê Bạch Mai</t>
+          <t>Nguyễn Xuân Ninh</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -1233,7 +1221,7 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Nguyên Phó Viện trưởng Viện Dinh dưỡng QG</t>
+          <t>Viện Y học Ứng dụng Việt Nam</t>
         </is>
       </c>
       <c r="F37">
@@ -1244,17 +1232,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>C04</t>
+          <t>C03</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đạo đức 1 (Bắt buộc)</t>
+          <t>Ủy viên Phản biện 2 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Thị Lâm</t>
+          <t>Lê Bạch Mai</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -1275,17 +1263,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>C05</t>
+          <t>C04</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đạo đức 2 (Bắt buộc)</t>
+          <t>Ủy viên HĐ Đạo đức 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Quang Dũng</t>
+          <t>Nguyễn Thị Lâm</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -1295,7 +1283,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Bộ môn Dinh dưỡng - ĐH Y Hà Nội</t>
+          <t>Nguyên Phó Viện trưởng Viện Dinh dưỡng QG</t>
         </is>
       </c>
       <c r="F39">
@@ -1306,28 +1294,43 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>C06</t>
+          <t>C05</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 3 (Tùy chọn)</t>
+          <t>Ủy viên HĐ Đạo đức 2 (Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Nguyễn Quang Dũng</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>PGS.TS.BS.</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Bộ môn Dinh dưỡng - ĐH Y Hà Nội</t>
         </is>
       </c>
       <c r="F40">
-        <f>IF(ISBLANK(C40), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C40), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>C07</t>
+          <t>C06</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đạo đức 3 (Tùy chọn)</t>
+          <t>Ủy viên Phản biện 3 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F41">
@@ -1338,12 +1341,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>C08</t>
+          <t>C07</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đạo đức 4 (Tùy chọn)</t>
+          <t>Ủy viên HĐ Đạo đức 3 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F42">
@@ -1354,48 +1357,33 @@
     <row r="43" ht="15" customHeight="1">
       <c r="A43" t="inlineStr">
         <is>
-          <t>C09</t>
+          <t>C08</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Thư ký HĐ Đạo đức 1 (Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>Hoàng Hà Linh</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="inlineStr">
-        <is>
-          <t>Thạc sĩ</t>
-        </is>
-      </c>
-      <c r="E43" s="3" t="inlineStr">
-        <is>
-          <t>Trung tâm NCKH - Viện VIAM</t>
+          <t>Ủy viên HĐ Đạo đức 4 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F43">
-        <f>IF(ISBLANK(C43), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C43), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>C10</t>
+          <t>C09</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Thư ký HĐ Đạo đức 2 (Bắt buộc)</t>
+          <t>Thư ký HĐ Đạo đức 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Trương Phan Hồng Hà</t>
+          <t>Hoàng Hà Linh</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -1405,7 +1393,7 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Viện Y học Ứng dụng Việt Nam</t>
+          <t>Trung tâm NCKH - Viện VIAM</t>
         </is>
       </c>
       <c r="F44">
@@ -1414,76 +1402,76 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Thư ký HĐ Đạo đức 2 (Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Trương Phan Hồng Hà</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Thạc sĩ</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>Viện Y học Ứng dụng Việt Nam</t>
+        </is>
+      </c>
+      <c r="F45">
+        <f>IF(ISBLANK(C45), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>SEC_D</t>
         </is>
       </c>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>PHẦN D: HỘI ĐỒNG KHOA HỌC XÉT DUYỆT ĐỀ CƯƠNG (HĐ 02 - 7 THÀNH VIÊN BẮT BUỘC)</t>
         </is>
       </c>
-      <c r="C45" s="2" t="n"/>
-      <c r="D45" s="2" t="n"/>
-      <c r="E45" s="2" t="n"/>
-      <c r="F45" s="2" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>D01</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Chủ tịch HĐ Đề cương (Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C46" s="3" t="inlineStr">
-        <is>
-          <t>Nguyễn Công Khẩn</t>
-        </is>
-      </c>
-      <c r="D46" s="3" t="inlineStr">
-        <is>
-          <t>GS.TS.</t>
-        </is>
-      </c>
-      <c r="E46" s="3" t="inlineStr">
-        <is>
-          <t>Hội đồng Đạo đức Y sinh Quốc gia</t>
-        </is>
-      </c>
-      <c r="F46">
-        <f>IF(ISBLANK(C46), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
-        <v/>
-      </c>
+      <c r="C46" s="2" t="n"/>
+      <c r="D46" s="2" t="n"/>
+      <c r="E46" s="2" t="n"/>
+      <c r="F46" s="2" t="n"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>D02</t>
+          <t>D01</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 1 (Bắt buộc)</t>
+          <t>Chủ tịch HĐ Đề cương (Bắt buộc)</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Xuân Ninh</t>
+          <t>Nguyễn Công Khẩn</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>PGS.TS.BS.</t>
+          <t>GS.TS.</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Viện Y học Ứng dụng Việt Nam</t>
+          <t>Hội đồng Đạo đức Y sinh Quốc gia</t>
         </is>
       </c>
       <c r="F47">
@@ -1494,27 +1482,27 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>D03</t>
+          <t>D02</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 2 (Bắt buộc)</t>
+          <t>Ủy viên Phản biện 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Trần Quang Trung</t>
+          <t>Nguyễn Xuân Ninh</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>PGS.TS.</t>
+          <t>PGS.TS.BS.</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Hiệp hội Sữa Việt Nam</t>
+          <t>Viện Y học Ứng dụng Việt Nam</t>
         </is>
       </c>
       <c r="F48">
@@ -1525,27 +1513,27 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>D04</t>
+          <t>D03</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đề cương 1 (Bắt buộc)</t>
+          <t>Ủy viên Phản biện 2 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Lê Bạch Mai</t>
+          <t>Trần Quang Trung</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>PGS.TS.BS.</t>
+          <t>PGS.TS.</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Nguyên Phó Viện trưởng Viện Dinh dưỡng QG</t>
+          <t>Hiệp hội Sữa Việt Nam</t>
         </is>
       </c>
       <c r="F49">
@@ -1556,17 +1544,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>D05</t>
+          <t>D04</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đề cương 2 (Bắt buộc)</t>
+          <t>Ủy viên HĐ Đề cương 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Thị Lâm</t>
+          <t>Lê Bạch Mai</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
@@ -1587,28 +1575,43 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>D06</t>
+          <t>D05</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 3 (Tùy chọn)</t>
+          <t>Ủy viên HĐ Đề cương 2 (Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Nguyễn Thị Lâm</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>PGS.TS.BS.</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Nguyên Phó Viện trưởng Viện Dinh dưỡng QG</t>
         </is>
       </c>
       <c r="F51">
-        <f>IF(ISBLANK(C51), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C51), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>D07</t>
+          <t>D06</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đề cương 3 (Tùy chọn)</t>
+          <t>Ủy viên Phản biện 3 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F52">
@@ -1619,12 +1622,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>D08</t>
+          <t>D07</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đề cương 4 (Tùy chọn)</t>
+          <t>Ủy viên HĐ Đề cương 3 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F53">
@@ -1635,48 +1638,33 @@
     <row r="54" ht="15" customHeight="1">
       <c r="A54" t="inlineStr">
         <is>
-          <t>D09</t>
+          <t>D08</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Thư ký HĐ Đề cương 1 (Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C54" s="3" t="inlineStr">
-        <is>
-          <t>Hoàng Hà Linh</t>
-        </is>
-      </c>
-      <c r="D54" s="3" t="inlineStr">
-        <is>
-          <t>Thạc sĩ</t>
-        </is>
-      </c>
-      <c r="E54" s="3" t="inlineStr">
-        <is>
-          <t>Trung tâm NCKH - Viện VIAM</t>
+          <t>Ủy viên HĐ Đề cương 4 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F54">
-        <f>IF(ISBLANK(C54), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C54), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>D09</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Thư ký HĐ Đề cương 2 (Bắt buộc)</t>
+          <t>Thư ký HĐ Đề cương 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Trương Phan Hồng Hà</t>
+          <t>Hoàng Hà Linh</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
@@ -1686,7 +1674,7 @@
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>Viện Y học Ứng dụng Việt Nam</t>
+          <t>Trung tâm NCKH - Viện VIAM</t>
         </is>
       </c>
       <c r="F55">
@@ -1695,76 +1683,76 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Thư ký HĐ Đề cương 2 (Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Trương Phan Hồng Hà</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>Thạc sĩ</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Viện Y học Ứng dụng Việt Nam</t>
+        </is>
+      </c>
+      <c r="F56">
+        <f>IF(ISBLANK(C56), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
         <is>
           <t>SEC_E</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="B57" s="2" t="inlineStr">
         <is>
           <t>PHẦN E: HỘI ĐỒNG ĐÁNH GIÁ NGHIỆM THU (HĐ 03 - 7 THÀNH VIÊN BẮT BUỘC)</t>
         </is>
       </c>
-      <c r="C56" s="2" t="n"/>
-      <c r="D56" s="2" t="n"/>
-      <c r="E56" s="2" t="n"/>
-      <c r="F56" s="2" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>E01</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Chủ tịch HĐ Nghiệm thu (Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C57" s="3" t="inlineStr">
-        <is>
-          <t>Phạm Văn Hoàn</t>
-        </is>
-      </c>
-      <c r="D57" s="3" t="inlineStr">
-        <is>
-          <t>PGS.TS.</t>
-        </is>
-      </c>
-      <c r="E57" s="3" t="inlineStr">
-        <is>
-          <t>Viện Y học Ứng dụng Việt Nam</t>
-        </is>
-      </c>
-      <c r="F57">
-        <f>IF(ISBLANK(C57), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
-        <v/>
-      </c>
+      <c r="C57" s="2" t="n"/>
+      <c r="D57" s="2" t="n"/>
+      <c r="E57" s="2" t="n"/>
+      <c r="F57" s="2" t="n"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>E02</t>
+          <t>E01</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 1 (Bắt buộc)</t>
+          <t>Chủ tịch HĐ Nghiệm thu (Bắt buộc)</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Công Khẩn</t>
+          <t>Phạm Văn Hoàn</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>GS.TS.</t>
+          <t>PGS.TS.</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>Hội đồng Đạo đức Y sinh Quốc gia</t>
+          <t>Viện Y học Ứng dụng Việt Nam</t>
         </is>
       </c>
       <c r="F58">
@@ -1775,27 +1763,27 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>E03</t>
+          <t>E02</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 2 (Bắt buộc)</t>
+          <t>Ủy viên Phản biện 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Nguyễn Thị Lâm</t>
+          <t>Nguyễn Công Khẩn</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>PGS.TS.BS.</t>
+          <t>GS.TS.</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>Nguyên Phó Viện trưởng Viện Dinh dưỡng QG</t>
+          <t>Hội đồng Đạo đức Y sinh Quốc gia</t>
         </is>
       </c>
       <c r="F59">
@@ -1806,27 +1794,27 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>E04</t>
+          <t>E03</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Nghiệm thu 1 (Bắt buộc)</t>
+          <t>Ủy viên Phản biện 2 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>Ninh Thị Nhung</t>
+          <t>Nguyễn Thị Lâm</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>PGS.TS.</t>
+          <t>PGS.TS.BS.</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>Trường Đại học Y Dược Thái Bình</t>
+          <t>Nguyên Phó Viện trưởng Viện Dinh dưỡng QG</t>
         </is>
       </c>
       <c r="F60">
@@ -1837,17 +1825,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>E05</t>
+          <t>E04</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Nghiệm thu 2 (Bắt buộc)</t>
+          <t>Ủy viên HĐ Nghiệm thu 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Trần Văn Ơn</t>
+          <t>Ninh Thị Nhung</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
@@ -1857,7 +1845,7 @@
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>Trường Đại học Dược Hà Nội</t>
+          <t>Trường Đại học Y Dược Thái Bình</t>
         </is>
       </c>
       <c r="F61">
@@ -1868,28 +1856,43 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>E06</t>
+          <t>E05</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 3 (Tùy chọn)</t>
+          <t>Ủy viên HĐ Nghiệm thu 2 (Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>Trần Văn Ơn</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>PGS.TS.</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>Trường Đại học Dược Hà Nội</t>
         </is>
       </c>
       <c r="F62">
-        <f>IF(ISBLANK(C62), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C62), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>E07</t>
+          <t>E06</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Nghiệm thu 3 (Tùy chọn)</t>
+          <t>Ủy viên Phản biện 3 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F63">
@@ -1900,12 +1903,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>E08</t>
+          <t>E07</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Nghiệm thu 4 (Tùy chọn)</t>
+          <t>Ủy viên HĐ Nghiệm thu 3 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F64">
@@ -1916,53 +1919,38 @@
     <row r="65" ht="15" customHeight="1">
       <c r="A65" t="inlineStr">
         <is>
-          <t>E09</t>
+          <t>E08</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Thư ký HĐ Nghiệm thu 1 (Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C65" s="3" t="inlineStr">
-        <is>
-          <t>Hoàng Hà Linh</t>
-        </is>
-      </c>
-      <c r="D65" s="3" t="inlineStr">
-        <is>
-          <t>PGS.TS.BS.</t>
-        </is>
-      </c>
-      <c r="E65" s="3" t="inlineStr">
-        <is>
-          <t>Viện Y học Ứng dụng Việt Nam</t>
+          <t>Ủy viên HĐ Nghiệm thu 4 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F65">
-        <f>IF(ISBLANK(C65), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C65), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>E10</t>
+          <t>E09</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Thư ký HĐ Nghiệm thu 2 (Bắt buộc)</t>
+          <t>Thư ký HĐ Nghiệm thu 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>Trương Phan Hồng Hà</t>
+          <t>Hoàng Hà Linh</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Thạc sĩ</t>
+          <t>PGS.TS.BS.</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
@@ -1976,77 +1964,92 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="inlineStr">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Thư ký HĐ Nghiệm thu 2 (Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>Trương Phan Hồng Hà</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Thạc sĩ</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>Viện Y học Ứng dụng Việt Nam</t>
+        </is>
+      </c>
+      <c r="F67">
+        <f>IF(ISBLANK(C67), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
         <is>
           <t>SEC_F</t>
         </is>
       </c>
-      <c r="B67" s="2" t="inlineStr">
+      <c r="B68" s="2" t="inlineStr">
         <is>
           <t>PHẦN F: LÝ LỊCH KHOA HỌC CHUYÊN GIA (CV CHỦ NHIỆM BẮT BUỘC &amp; CV THÀNH VIÊN TÙY CHỌN)</t>
         </is>
       </c>
-      <c r="C67" s="2" t="n"/>
-      <c r="D67" s="2" t="n"/>
-      <c r="E67" s="2" t="n"/>
-      <c r="F67" s="2" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>F01</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>Hồ sơ Chủ nhiệm đề tài (Bắt buộc - File mặc định cho HĐ Đạo đức)</t>
-        </is>
-      </c>
-      <c r="C68" s="3" t="inlineStr">
-        <is>
-          <t>Trương Hồng Sơn</t>
-        </is>
-      </c>
-      <c r="D68" s="3" t="inlineStr">
-        <is>
-          <t>Chủ nhiệm đề tài</t>
-        </is>
-      </c>
-      <c r="E68" s="3" t="inlineStr">
-        <is>
-          <t>Lý lịch khoa học - Trương Hồng Sơn.docx</t>
-        </is>
-      </c>
-      <c r="F68">
-        <f>IF(ISBLANK(C68), "❌ CHƯA ĐIỀN THÔNG TIN CNĐT (BÁO LỖI)", IF(OR(ISBLANK(D68), ISBLANK(E68)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV Mặc định Đạo đức"))</f>
-        <v/>
-      </c>
+      <c r="C68" s="2" t="n"/>
+      <c r="D68" s="2" t="n"/>
+      <c r="E68" s="2" t="n"/>
+      <c r="F68" s="2" t="n"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>F02</t>
+          <t>F01</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Hồ sơ Đồng Chủ nhiệm (Tùy chọn)</t>
+          <t>Hồ sơ Chủ nhiệm đề tài (Bắt buộc - File mặc định cho HĐ Đạo đức)</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>Trương Hồng Sơn</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>Chủ nhiệm đề tài</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>Lý lịch khoa học - Trương Hồng Sơn.docx</t>
         </is>
       </c>
       <c r="F69">
-        <f>IF(ISBLANK(C69), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D69), ISBLANK(E69)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
+        <f>IF(ISBLANK(C69), "❌ CHƯA ĐIỀN THÔNG TIN CNĐT (BÁO LỖI)", IF(OR(ISBLANK(D69), ISBLANK(E69)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV Mặc định Đạo đức"))</f>
         <v/>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>F03</t>
+          <t>F02</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Hồ sơ Thư ký Đề tài (Tùy chọn)</t>
+          <t>Hồ sơ Đồng Chủ nhiệm (Tùy chọn)</t>
         </is>
       </c>
       <c r="F70">
@@ -2057,27 +2060,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>F04</t>
+          <t>F03</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 4 (Tùy chọn)</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>Nguyễn Công Khẩn</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>Chuyên gia hội đồng</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>TM-Gs. Nguyen Cong Khan.pdf</t>
+          <t>Hồ sơ Thư ký Đề tài (Tùy chọn)</t>
         </is>
       </c>
       <c r="F71">
@@ -2088,17 +2076,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>F05</t>
+          <t>F04</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 5 (Tùy chọn)</t>
+          <t>Hồ sơ Chuyên gia / Thành viên 4 (Tùy chọn)</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Hoàng Thị Thanh</t>
+          <t>Nguyễn Công Khẩn</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2108,7 +2096,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>TM-PGs. Hoang Thi Thanh.pdf</t>
+          <t>TM-Gs. Nguyen Cong Khan.pdf</t>
         </is>
       </c>
       <c r="F72">
@@ -2119,17 +2107,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>F06</t>
+          <t>F05</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 6 (Tùy chọn)</t>
+          <t>Hồ sơ Chuyên gia / Thành viên 5 (Tùy chọn)</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Nguyễn Quang Dũng</t>
+          <t>Hoàng Thị Thanh</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2139,7 +2127,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>TM-PGs. Nguyen Quang Dung.pdf</t>
+          <t>TM-PGs. Hoang Thi Thanh.pdf</t>
         </is>
       </c>
       <c r="F73">
@@ -2150,17 +2138,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>F07</t>
+          <t>F06</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 7 (Tùy chọn)</t>
+          <t>Hồ sơ Chuyên gia / Thành viên 6 (Tùy chọn)</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Trần Quang Trung</t>
+          <t>Nguyễn Quang Dũng</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2170,7 +2158,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>TM-PGs. Tran Quang Trung.pdf</t>
+          <t>TM-PGs. Nguyen Quang Dung.pdf</t>
         </is>
       </c>
       <c r="F74">
@@ -2181,17 +2169,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>F08</t>
+          <t>F07</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 8 (Tùy chọn)</t>
+          <t>Hồ sơ Chuyên gia / Thành viên 7 (Tùy chọn)</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Nguyễn Hùng Long</t>
+          <t>Trần Quang Trung</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2201,7 +2189,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>TM-Ts. Nguyen Hung Long.pdf</t>
+          <t>TM-PGs. Tran Quang Trung.pdf</t>
         </is>
       </c>
       <c r="F75">
@@ -2212,12 +2200,27 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>F09</t>
+          <t>F08</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 9 (Tùy chọn)</t>
+          <t>Hồ sơ Chuyên gia / Thành viên 8 (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Nguyễn Hùng Long</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Chuyên gia hội đồng</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>TM-Ts. Nguyen Hung Long.pdf</t>
         </is>
       </c>
       <c r="F76">
@@ -2228,16 +2231,32 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>F10</t>
+          <t>F09</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 10 (Tùy chọn)</t>
+          <t>Hồ sơ Chuyên gia / Thành viên 9 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F77">
         <f>IF(ISBLANK(C77), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D77), ISBLANK(E77)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>F10</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Hồ sơ Chuyên gia / Thành viên 10 (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="F78">
+        <f>IF(ISBLANK(C78), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D78), ISBLANK(E78)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
         <v/>
       </c>
     </row>
@@ -2256,7 +2275,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F77"/>
+  <dimension ref="A1:F78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="8.5" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2462,65 +2481,68 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>A08</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Đầu mối liên hệ (họ tên, đơn vị, email, điện thoại - Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n"/>
+      <c r="D13" s="3" t="n"/>
+      <c r="E13" s="3" t="n"/>
+      <c r="F13">
+        <f>IF(ISBLANK(C13), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>SEC_B</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>PHẦN B: BAN CHỦ NHIỆM &amp; NGHIÊN CỨU VIÊN ĐỀ TÀI (TỐI ĐA 20 NGƯỜI)</t>
         </is>
       </c>
-      <c r="C13" s="2" t="n"/>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>B01</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Chủ nhiệm đề tài (CNĐT - Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14">
-        <f>IF(ISBLANK(C14), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
-        <v/>
-      </c>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>B02</t>
+          <t>B01</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Đồng Chủ nhiệm đề tài (Tùy chọn)</t>
-        </is>
-      </c>
+          <t>Chủ nhiệm đề tài (CNĐT - Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="3" t="n"/>
       <c r="F15">
-        <f>IF(ISBLANK(C15), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C15), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>B03</t>
+          <t>B02</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Thư ký Đề tài (Khác Thư ký HĐ - Tùy chọn)</t>
+          <t>Đồng Chủ nhiệm đề tài (Tùy chọn)</t>
         </is>
       </c>
       <c r="F16">
@@ -2531,12 +2553,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>B04</t>
+          <t>B03</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 1</t>
+          <t>Thư ký Đề tài (Khác Thư ký HĐ - Tùy chọn)</t>
         </is>
       </c>
       <c r="F17">
@@ -2547,12 +2569,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>B05</t>
+          <t>B04</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 2</t>
+          <t>Nghiên cứu viên 1</t>
         </is>
       </c>
       <c r="F18">
@@ -2563,12 +2585,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>B06</t>
+          <t>B05</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 3</t>
+          <t>Nghiên cứu viên 2</t>
         </is>
       </c>
       <c r="F19">
@@ -2579,12 +2601,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>B07</t>
+          <t>B06</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 4</t>
+          <t>Nghiên cứu viên 3</t>
         </is>
       </c>
       <c r="F20">
@@ -2595,12 +2617,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>B08</t>
+          <t>B07</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 5</t>
+          <t>Nghiên cứu viên 4</t>
         </is>
       </c>
       <c r="F21">
@@ -2611,12 +2633,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>B09</t>
+          <t>B08</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 6</t>
+          <t>Nghiên cứu viên 5</t>
         </is>
       </c>
       <c r="F22">
@@ -2627,12 +2649,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>B10</t>
+          <t>B09</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 7</t>
+          <t>Nghiên cứu viên 6</t>
         </is>
       </c>
       <c r="F23">
@@ -2643,12 +2665,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>B11</t>
+          <t>B10</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 8</t>
+          <t>Nghiên cứu viên 7</t>
         </is>
       </c>
       <c r="F24">
@@ -2659,12 +2681,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>B12</t>
+          <t>B11</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 9</t>
+          <t>Nghiên cứu viên 8</t>
         </is>
       </c>
       <c r="F25">
@@ -2675,12 +2697,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>B13</t>
+          <t>B12</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 10</t>
+          <t>Nghiên cứu viên 9</t>
         </is>
       </c>
       <c r="F26">
@@ -2691,12 +2713,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>B14</t>
+          <t>B13</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 11</t>
+          <t>Nghiên cứu viên 10</t>
         </is>
       </c>
       <c r="F27">
@@ -2707,12 +2729,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>B15</t>
+          <t>B14</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 12</t>
+          <t>Nghiên cứu viên 11</t>
         </is>
       </c>
       <c r="F28">
@@ -2723,12 +2745,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>B16</t>
+          <t>B15</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 13</t>
+          <t>Nghiên cứu viên 12</t>
         </is>
       </c>
       <c r="F29">
@@ -2739,12 +2761,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>B17</t>
+          <t>B16</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 14</t>
+          <t>Nghiên cứu viên 13</t>
         </is>
       </c>
       <c r="F30">
@@ -2755,12 +2777,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>B18</t>
+          <t>B17</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 15</t>
+          <t>Nghiên cứu viên 14</t>
         </is>
       </c>
       <c r="F31">
@@ -2771,17 +2793,12 @@
     <row r="32" ht="15" customHeight="1">
       <c r="A32" t="inlineStr">
         <is>
-          <t>B19</t>
+          <t>B18</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 16</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>(Để trống tên theo quy định)</t>
+          <t>Nghiên cứu viên 15</t>
         </is>
       </c>
       <c r="F32">
@@ -2792,12 +2809,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>B20</t>
+          <t>B19</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Nghiên cứu viên 17</t>
+          <t>Nghiên cứu viên 16</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2811,49 +2828,51 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>B20</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Nghiên cứu viên 17</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>(Để trống tên theo quy định)</t>
+        </is>
+      </c>
+      <c r="F34">
+        <f>IF(ISBLANK(C34), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>SEC_C</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>PHẦN C: HỘI ĐỒNG ĐẠO ĐỨC TRONG NGHIÊN CỨU (HĐ 01 - 7 THÀNH VIÊN BẮT BUỘC)</t>
         </is>
       </c>
-      <c r="C34" s="2" t="n"/>
-      <c r="D34" s="2" t="n"/>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="2" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>C01</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Chủ tịch HĐ Đạo đức (Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="n"/>
-      <c r="D35" s="3" t="n"/>
-      <c r="E35" s="3" t="n"/>
-      <c r="F35">
-        <f>IF(ISBLANK(C35), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
-        <v/>
-      </c>
+      <c r="C35" s="2" t="n"/>
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>C02</t>
+          <t>C01</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 1 (Bắt buộc)</t>
+          <t>Chủ tịch HĐ Đạo đức (Bắt buộc)</t>
         </is>
       </c>
       <c r="C36" s="3" t="n"/>
@@ -2867,12 +2886,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>C03</t>
+          <t>C02</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 2 (Bắt buộc)</t>
+          <t>Ủy viên Phản biện 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C37" s="3" t="n"/>
@@ -2886,12 +2905,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>C04</t>
+          <t>C03</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đạo đức 1 (Bắt buộc)</t>
+          <t>Ủy viên Phản biện 2 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C38" s="3" t="n"/>
@@ -2905,12 +2924,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>C05</t>
+          <t>C04</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đạo đức 2 (Bắt buộc)</t>
+          <t>Ủy viên HĐ Đạo đức 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C39" s="3" t="n"/>
@@ -2924,28 +2943,31 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>C06</t>
+          <t>C05</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 3 (Tùy chọn)</t>
-        </is>
-      </c>
+          <t>Ủy viên HĐ Đạo đức 2 (Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="n"/>
+      <c r="D40" s="3" t="n"/>
+      <c r="E40" s="3" t="n"/>
       <c r="F40">
-        <f>IF(ISBLANK(C40), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C40), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>C07</t>
+          <t>C06</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đạo đức 3 (Tùy chọn)</t>
+          <t>Ủy viên Phản biện 3 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F41">
@@ -2956,12 +2978,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>C08</t>
+          <t>C07</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đạo đức 4 (Tùy chọn)</t>
+          <t>Ủy viên HĐ Đạo đức 3 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F42">
@@ -2972,31 +2994,28 @@
     <row r="43" ht="15" customHeight="1">
       <c r="A43" t="inlineStr">
         <is>
-          <t>C09</t>
+          <t>C08</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Thư ký HĐ Đạo đức 1 (Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="n"/>
-      <c r="D43" s="3" t="n"/>
-      <c r="E43" s="3" t="n"/>
+          <t>Ủy viên HĐ Đạo đức 4 (Tùy chọn)</t>
+        </is>
+      </c>
       <c r="F43">
-        <f>IF(ISBLANK(C43), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C43), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>C10</t>
+          <t>C09</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Thư ký HĐ Đạo đức 2 (Bắt buộc)</t>
+          <t>Thư ký HĐ Đạo đức 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C44" s="3" t="n"/>
@@ -3008,49 +3027,49 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Thư ký HĐ Đạo đức 2 (Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="n"/>
+      <c r="D45" s="3" t="n"/>
+      <c r="E45" s="3" t="n"/>
+      <c r="F45">
+        <f>IF(ISBLANK(C45), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>SEC_D</t>
         </is>
       </c>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>PHẦN D: HỘI ĐỒNG KHOA HỌC XÉT DUYỆT ĐỀ CƯƠNG (HĐ 02 - 7 THÀNH VIÊN BẮT BUỘC)</t>
         </is>
       </c>
-      <c r="C45" s="2" t="n"/>
-      <c r="D45" s="2" t="n"/>
-      <c r="E45" s="2" t="n"/>
-      <c r="F45" s="2" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>D01</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Chủ tịch HĐ Đề cương (Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C46" s="3" t="n"/>
-      <c r="D46" s="3" t="n"/>
-      <c r="E46" s="3" t="n"/>
-      <c r="F46">
-        <f>IF(ISBLANK(C46), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
-        <v/>
-      </c>
+      <c r="C46" s="2" t="n"/>
+      <c r="D46" s="2" t="n"/>
+      <c r="E46" s="2" t="n"/>
+      <c r="F46" s="2" t="n"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>D02</t>
+          <t>D01</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 1 (Bắt buộc)</t>
+          <t>Chủ tịch HĐ Đề cương (Bắt buộc)</t>
         </is>
       </c>
       <c r="C47" s="3" t="n"/>
@@ -3064,12 +3083,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>D03</t>
+          <t>D02</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 2 (Bắt buộc)</t>
+          <t>Ủy viên Phản biện 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C48" s="3" t="n"/>
@@ -3083,12 +3102,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>D04</t>
+          <t>D03</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đề cương 1 (Bắt buộc)</t>
+          <t>Ủy viên Phản biện 2 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C49" s="3" t="n"/>
@@ -3102,12 +3121,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>D05</t>
+          <t>D04</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đề cương 2 (Bắt buộc)</t>
+          <t>Ủy viên HĐ Đề cương 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C50" s="3" t="n"/>
@@ -3121,28 +3140,31 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>D06</t>
+          <t>D05</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 3 (Tùy chọn)</t>
-        </is>
-      </c>
+          <t>Ủy viên HĐ Đề cương 2 (Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="n"/>
+      <c r="D51" s="3" t="n"/>
+      <c r="E51" s="3" t="n"/>
       <c r="F51">
-        <f>IF(ISBLANK(C51), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C51), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>D07</t>
+          <t>D06</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đề cương 3 (Tùy chọn)</t>
+          <t>Ủy viên Phản biện 3 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F52">
@@ -3153,12 +3175,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>D08</t>
+          <t>D07</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Đề cương 4 (Tùy chọn)</t>
+          <t>Ủy viên HĐ Đề cương 3 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F53">
@@ -3169,31 +3191,28 @@
     <row r="54" ht="15" customHeight="1">
       <c r="A54" t="inlineStr">
         <is>
-          <t>D09</t>
+          <t>D08</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Thư ký HĐ Đề cương 1 (Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C54" s="3" t="n"/>
-      <c r="D54" s="3" t="n"/>
-      <c r="E54" s="3" t="n"/>
+          <t>Ủy viên HĐ Đề cương 4 (Tùy chọn)</t>
+        </is>
+      </c>
       <c r="F54">
-        <f>IF(ISBLANK(C54), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C54), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>D09</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Thư ký HĐ Đề cương 2 (Bắt buộc)</t>
+          <t>Thư ký HĐ Đề cương 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C55" s="3" t="n"/>
@@ -3205,49 +3224,49 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Thư ký HĐ Đề cương 2 (Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="n"/>
+      <c r="D56" s="3" t="n"/>
+      <c r="E56" s="3" t="n"/>
+      <c r="F56">
+        <f>IF(ISBLANK(C56), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
         <is>
           <t>SEC_E</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="B57" s="2" t="inlineStr">
         <is>
           <t>PHẦN E: HỘI ĐỒNG ĐÁNH GIÁ NGHIỆM THU (HĐ 03 - 7 THÀNH VIÊN BẮT BUỘC)</t>
         </is>
       </c>
-      <c r="C56" s="2" t="n"/>
-      <c r="D56" s="2" t="n"/>
-      <c r="E56" s="2" t="n"/>
-      <c r="F56" s="2" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>E01</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Chủ tịch HĐ Nghiệm thu (Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C57" s="3" t="n"/>
-      <c r="D57" s="3" t="n"/>
-      <c r="E57" s="3" t="n"/>
-      <c r="F57">
-        <f>IF(ISBLANK(C57), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
-        <v/>
-      </c>
+      <c r="C57" s="2" t="n"/>
+      <c r="D57" s="2" t="n"/>
+      <c r="E57" s="2" t="n"/>
+      <c r="F57" s="2" t="n"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>E02</t>
+          <t>E01</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 1 (Bắt buộc)</t>
+          <t>Chủ tịch HĐ Nghiệm thu (Bắt buộc)</t>
         </is>
       </c>
       <c r="C58" s="3" t="n"/>
@@ -3261,12 +3280,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>E03</t>
+          <t>E02</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 2 (Bắt buộc)</t>
+          <t>Ủy viên Phản biện 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C59" s="3" t="n"/>
@@ -3280,12 +3299,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>E04</t>
+          <t>E03</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Nghiệm thu 1 (Bắt buộc)</t>
+          <t>Ủy viên Phản biện 2 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C60" s="3" t="n"/>
@@ -3299,12 +3318,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>E05</t>
+          <t>E04</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Nghiệm thu 2 (Bắt buộc)</t>
+          <t>Ủy viên HĐ Nghiệm thu 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C61" s="3" t="n"/>
@@ -3318,28 +3337,31 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>E06</t>
+          <t>E05</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Ủy viên Phản biện 3 (Tùy chọn)</t>
-        </is>
-      </c>
+          <t>Ủy viên HĐ Nghiệm thu 2 (Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="n"/>
+      <c r="D62" s="3" t="n"/>
+      <c r="E62" s="3" t="n"/>
       <c r="F62">
-        <f>IF(ISBLANK(C62), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C62), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>E07</t>
+          <t>E06</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Nghiệm thu 3 (Tùy chọn)</t>
+          <t>Ủy viên Phản biện 3 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F63">
@@ -3350,12 +3372,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>E08</t>
+          <t>E07</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Ủy viên HĐ Nghiệm thu 4 (Tùy chọn)</t>
+          <t>Ủy viên HĐ Nghiệm thu 3 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F64">
@@ -3366,31 +3388,28 @@
     <row r="65" ht="15" customHeight="1">
       <c r="A65" t="inlineStr">
         <is>
-          <t>E09</t>
+          <t>E08</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Thư ký HĐ Nghiệm thu 1 (Bắt buộc)</t>
-        </is>
-      </c>
-      <c r="C65" s="3" t="n"/>
-      <c r="D65" s="3" t="n"/>
-      <c r="E65" s="3" t="n"/>
+          <t>Ủy viên HĐ Nghiệm thu 4 (Tùy chọn)</t>
+        </is>
+      </c>
       <c r="F65">
-        <f>IF(ISBLANK(C65), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
+        <f>IF(ISBLANK(C65), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
         <v/>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>E10</t>
+          <t>E09</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Thư ký HĐ Nghiệm thu 2 (Bắt buộc)</t>
+          <t>Thư ký HĐ Nghiệm thu 1 (Bắt buộc)</t>
         </is>
       </c>
       <c r="C66" s="3" t="n"/>
@@ -3402,65 +3421,68 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="inlineStr">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Thư ký HĐ Nghiệm thu 2 (Bắt buộc)</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="n"/>
+      <c r="D67" s="3" t="n"/>
+      <c r="E67" s="3" t="n"/>
+      <c r="F67">
+        <f>IF(ISBLANK(C67), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
         <is>
           <t>SEC_F</t>
         </is>
       </c>
-      <c r="B67" s="2" t="inlineStr">
+      <c r="B68" s="2" t="inlineStr">
         <is>
           <t>PHẦN F: LÝ LỊCH KHOA HỌC CHUYÊN GIA (CV CHỦ NHIỆM BẮT BUỘC &amp; CV THÀNH VIÊN TÙY CHỌN)</t>
         </is>
       </c>
-      <c r="C67" s="2" t="n"/>
-      <c r="D67" s="2" t="n"/>
-      <c r="E67" s="2" t="n"/>
-      <c r="F67" s="2" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>F01</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>Hồ sơ Chủ nhiệm đề tài (Bắt buộc - File mặc định cho HĐ Đạo đức)</t>
-        </is>
-      </c>
-      <c r="C68" s="3" t="n"/>
-      <c r="D68" s="3" t="n"/>
-      <c r="E68" s="3" t="n"/>
-      <c r="F68">
-        <f>IF(ISBLANK(C68), "❌ CHƯA ĐIỀN THÔNG TIN CNĐT (BÁO LỖI)", IF(OR(ISBLANK(D68), ISBLANK(E68)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV Mặc định Đạo đức"))</f>
-        <v/>
-      </c>
+      <c r="C68" s="2" t="n"/>
+      <c r="D68" s="2" t="n"/>
+      <c r="E68" s="2" t="n"/>
+      <c r="F68" s="2" t="n"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>F02</t>
+          <t>F01</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Hồ sơ Đồng Chủ nhiệm (Tùy chọn)</t>
-        </is>
-      </c>
+          <t>Hồ sơ Chủ nhiệm đề tài (Bắt buộc - File mặc định cho HĐ Đạo đức)</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="n"/>
+      <c r="D69" s="3" t="n"/>
+      <c r="E69" s="3" t="n"/>
       <c r="F69">
-        <f>IF(ISBLANK(C69), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D69), ISBLANK(E69)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
+        <f>IF(ISBLANK(C69), "❌ CHƯA ĐIỀN THÔNG TIN CNĐT (BÁO LỖI)", IF(OR(ISBLANK(D69), ISBLANK(E69)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV Mặc định Đạo đức"))</f>
         <v/>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>F03</t>
+          <t>F02</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Hồ sơ Thư ký Đề tài (Tùy chọn)</t>
+          <t>Hồ sơ Đồng Chủ nhiệm (Tùy chọn)</t>
         </is>
       </c>
       <c r="F70">
@@ -3471,12 +3493,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>F04</t>
+          <t>F03</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 4 (Tùy chọn)</t>
+          <t>Hồ sơ Thư ký Đề tài (Tùy chọn)</t>
         </is>
       </c>
       <c r="F71">
@@ -3487,12 +3509,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>F05</t>
+          <t>F04</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 5 (Tùy chọn)</t>
+          <t>Hồ sơ Chuyên gia / Thành viên 4 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F72">
@@ -3503,12 +3525,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>F06</t>
+          <t>F05</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 6 (Tùy chọn)</t>
+          <t>Hồ sơ Chuyên gia / Thành viên 5 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F73">
@@ -3519,12 +3541,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>F07</t>
+          <t>F06</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 7 (Tùy chọn)</t>
+          <t>Hồ sơ Chuyên gia / Thành viên 6 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F74">
@@ -3535,12 +3557,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>F08</t>
+          <t>F07</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 8 (Tùy chọn)</t>
+          <t>Hồ sơ Chuyên gia / Thành viên 7 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F75">
@@ -3551,12 +3573,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>F09</t>
+          <t>F08</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 9 (Tùy chọn)</t>
+          <t>Hồ sơ Chuyên gia / Thành viên 8 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F76">
@@ -3567,16 +3589,32 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>F10</t>
+          <t>F09</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Hồ sơ Chuyên gia / Thành viên 10 (Tùy chọn)</t>
+          <t>Hồ sơ Chuyên gia / Thành viên 9 (Tùy chọn)</t>
         </is>
       </c>
       <c r="F77">
         <f>IF(ISBLANK(C77), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D77), ISBLANK(E77)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>F10</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Hồ sơ Chuyên gia / Thành viên 10 (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="F78">
+        <f>IF(ISBLANK(C78), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D78), ISBLANK(E78)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
         <v/>
       </c>
     </row>
@@ -3659,302 +3697,313 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>token_name</t>
+          <t>ten</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>code</t>
+          <t>hoc_ham_hoc_vi</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>kind</t>
+          <t>don_vi</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>param</t>
+          <t>dia_chi</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>sdt</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>cccd</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>mst</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>so_tk</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>ngan_hang</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TEN_DE_TAI</t>
+          <t>Trương Hồng Sơn</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>A01</t>
+          <t>TS.BS.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>raw</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Tên đề tài</t>
+          <t>Viện trưởng - Viện Y học Ứng dụng VN</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>NAM</t>
+          <t>Lưu Liên Hương</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>A03</t>
+          <t>Thạc sĩ</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>raw</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Năm thực hiện hồ sơ</t>
+          <t>Trung tâm NCKH - Viện VIAM</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DON_VI_CHU_TRI</t>
+          <t>Lê Việt Anh</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>A04</t>
+          <t>Thạc sĩ</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>raw</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Cơ quan chủ trì</t>
+          <t>Trung tâm NCKH - Viện VIAM</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DON_VI_DOI_TAC</t>
+          <t>Lê Minh Khánh</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>A06</t>
+          <t>Bác sĩ</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>raw</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Cơ quan phối hợp</t>
+          <t>Phòng khám VIAM</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CHU_NHIEM_HO_TEN</t>
+          <t>Nguyễn Công Khẩn</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>B01</t>
+          <t>GS.TS.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>person_ho_ten</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Chủ nhiệm đề tài - có học hàm/học vị</t>
+          <t>Hội đồng Đạo đức Y sinh Quốc gia</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CHU_NHIEM_TEN</t>
+          <t>Nguyễn Xuân Ninh</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>B01</t>
+          <t>PGS.TS.BS.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>person_ten</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Chủ nhiệm đề tài - chỉ tên</t>
+          <t>Viện Y học Ứng dụng Việt Nam</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DONG_CHU_NHIEM_TEN</t>
+          <t>Lê Bạch Mai</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>B02</t>
+          <t>PGS.TS.BS.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>person_ten</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Đồng chủ nhiệm đề tài - chỉ tên</t>
+          <t>Nguyên Phó Viện trưởng Viện Dinh dưỡng QG</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DONG_CHU_NHIEM_HO_TEN</t>
+          <t>Nguyễn Thị Lâm</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>B02</t>
+          <t>PGS.TS.BS.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>person_ho_ten</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Đồng chủ nhiệm đề tài - có học hàm/học vị</t>
+          <t>Nguyên Phó Viện trưởng Viện Dinh dưỡng QG</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>THU_KY_DE_TAI</t>
+          <t>Nguyễn Quang Dũng</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>B03</t>
+          <t>PGS.TS.BS.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>person_ho_ten</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Thư ký đề tài</t>
+          <t>Bộ môn Dinh dưỡng - ĐH Y Hà Nội</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>THOI_GIAN_BAT_DAU</t>
+          <t>Hoàng Hà Linh</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A05</t>
+          <t>Thạc sĩ</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>timeline_start</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Mốc bắt đầu (MM/YYYY)</t>
+          <t>Trung tâm NCKH - Viện VIAM</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>THOI_GIAN_KET_THUC</t>
+          <t>Trương Phan Hồng Hà</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>A05</t>
+          <t>Thạc sĩ</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>timeline_end</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Mốc kết thúc (MM/YYYY)</t>
+          <t>Viện Y học Ứng dụng Việt Nam</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DIA_DIEM_TRIEN_KHAI</t>
+          <t>Trần Quang Trung</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>A07</t>
+          <t>PGS.TS.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>raw_or_placeholder</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>……………………………</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Địa điểm triển khai nghiên cứu</t>
+          <t>Hiệp hội Sữa Việt Nam</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Phạm Văn Hoàn</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PGS.TS.</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Viện Y học Ứng dụng Việt Nam</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Ninh Thị Nhung</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>PGS.TS.</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Trường Đại học Y Dược Thái Bình</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Trần Văn Ơn</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>PGS.TS.</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Trường Đại học Dược Hà Nội</t>
         </is>
       </c>
     </row>
@@ -3969,313 +4018,340 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>ten</t>
+          <t>token_name</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>hoc_ham_hoc_vi</t>
+          <t>code</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>don_vi</t>
+          <t>kind</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>dia_chi</t>
+          <t>param</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>sdt</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>email</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>cccd</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>mst</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>so_tk</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>ngan_hang</t>
+          <t>note</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Trương Hồng Sơn</t>
+          <t>TEN_DE_TAI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>TS.BS.</t>
+          <t>A01</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Viện trưởng - Viện Y học Ứng dụng VN</t>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Tên đề tài</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Lưu Liên Hương</t>
+          <t>NAM</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Thạc sĩ</t>
+          <t>A03</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Trung tâm NCKH - Viện VIAM</t>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Năm thực hiện hồ sơ</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lê Việt Anh</t>
+          <t>DON_VI_CHU_TRI</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Thạc sĩ</t>
+          <t>A04</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Trung tâm NCKH - Viện VIAM</t>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Cơ quan chủ trì</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Lê Minh Khánh</t>
+          <t>DON_VI_DOI_TAC</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Bác sĩ</t>
+          <t>A06</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Phòng khám VIAM</t>
+          <t>raw_or_placeholder</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Cơ quan phối hợp</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Nguyễn Công Khẩn</t>
+          <t>CHU_NHIEM_HO_TEN</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>GS.TS.</t>
+          <t>B01</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Hội đồng Đạo đức Y sinh Quốc gia</t>
+          <t>person_ho_ten</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Chủ nhiệm đề tài - có học hàm/học vị</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Nguyễn Xuân Ninh</t>
+          <t>CHU_NHIEM_TEN</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PGS.TS.BS.</t>
+          <t>B01</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Viện Y học Ứng dụng Việt Nam</t>
+          <t>person_ten</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Chủ nhiệm đề tài - chỉ tên</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Lê Bạch Mai</t>
+          <t>DONG_CHU_NHIEM_TEN</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PGS.TS.BS.</t>
+          <t>B02</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Nguyên Phó Viện trưởng Viện Dinh dưỡng QG</t>
+          <t>person_ten</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Đồng chủ nhiệm đề tài - chỉ tên</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Nguyễn Thị Lâm</t>
+          <t>DONG_CHU_NHIEM_HO_TEN</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PGS.TS.BS.</t>
+          <t>B02</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Nguyên Phó Viện trưởng Viện Dinh dưỡng QG</t>
+          <t>person_ho_ten</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Đồng chủ nhiệm đề tài - có học hàm/học vị</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Nguyễn Quang Dũng</t>
+          <t>THU_KY_DE_TAI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PGS.TS.BS.</t>
+          <t>B03</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Bộ môn Dinh dưỡng - ĐH Y Hà Nội</t>
+          <t>person_ho_ten</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Thư ký đề tài</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Hoàng Hà Linh</t>
+          <t>THOI_GIAN_BAT_DAU</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Thạc sĩ</t>
+          <t>A05</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Trung tâm NCKH - Viện VIAM</t>
+          <t>timeline_start</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Mốc bắt đầu (MM/YYYY)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Trương Phan Hồng Hà</t>
+          <t>THOI_GIAN_KET_THUC</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Thạc sĩ</t>
+          <t>A05</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Viện Y học Ứng dụng Việt Nam</t>
+          <t>timeline_end</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Mốc kết thúc (MM/YYYY)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Trần Quang Trung</t>
+          <t>DIA_DIEM_TRIEN_KHAI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PGS.TS.</t>
+          <t>A07</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Hiệp hội Sữa Việt Nam</t>
+          <t>raw_or_placeholder</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>……………………………</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Địa điểm triển khai nghiên cứu</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Phạm Văn Hoàn</t>
+          <t>DAU_MOI_LIEN_HE</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PGS.TS.</t>
+          <t>A08</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Viện Y học Ứng dụng Việt Nam</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Ninh Thị Nhung</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>PGS.TS.</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Trường Đại học Y Dược Thái Bình</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Trần Văn Ơn</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>PGS.TS.</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Trường Đại học Dược Hà Nội</t>
+          <t>raw_or_placeholder</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>……</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Đầu mối liên hệ (thư mời chuyên gia)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: remove CV-filename dropdown/validation, retire its refresh script
</commit_message>
<xml_diff>
--- a/Form checklist hồ sơ dự án.xlsx
+++ b/Form checklist hồ sơ dự án.xlsx
@@ -8,9 +8,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đề tài - Bánh ăn dặm VIAM 2027" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đề tài - Mẫu trắng dự án mới" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Lists" sheetId="3" state="hidden" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_NhanSu" sheetId="4" state="hidden" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Tokens" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_NhanSu" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Tokens" sheetId="4" state="hidden" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -2037,7 +2036,7 @@
         </is>
       </c>
       <c r="F69">
-        <f>IF(ISBLANK(C69), "❌ CHƯA ĐIỀN THÔNG TIN CNĐT (BÁO LỖI)", IF(OR(ISBLANK(D69), ISBLANK(E69)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV Mặc định Đạo đức"))</f>
+        <f>IF(ISBLANK(C69), "❌ CHƯA ĐIỀN THÔNG TIN CNĐT (BÁO LỖI)", "✅ Đã khai chủ nhiệm đề tài - CV sẽ tự khớp theo tên")</f>
         <v/>
       </c>
     </row>
@@ -2053,7 +2052,7 @@
         </is>
       </c>
       <c r="F70">
-        <f>IF(ISBLANK(C70), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D70), ISBLANK(E70)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
+        <f>IF(ISBLANK(C70), "⚪ Tùy chọn (Trống)", "✅ Đã khai tên - CV sẽ tự khớp theo tên")</f>
         <v/>
       </c>
     </row>
@@ -2069,7 +2068,7 @@
         </is>
       </c>
       <c r="F71">
-        <f>IF(ISBLANK(C71), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D71), ISBLANK(E71)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
+        <f>IF(ISBLANK(C71), "⚪ Tùy chọn (Trống)", "✅ Đã khai tên - CV sẽ tự khớp theo tên")</f>
         <v/>
       </c>
     </row>
@@ -2100,7 +2099,7 @@
         </is>
       </c>
       <c r="F72">
-        <f>IF(ISBLANK(C72), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D72), ISBLANK(E72)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
+        <f>IF(ISBLANK(C72), "⚪ Tùy chọn (Trống)", "✅ Đã khai tên - CV sẽ tự khớp theo tên")</f>
         <v/>
       </c>
     </row>
@@ -2131,7 +2130,7 @@
         </is>
       </c>
       <c r="F73">
-        <f>IF(ISBLANK(C73), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D73), ISBLANK(E73)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
+        <f>IF(ISBLANK(C73), "⚪ Tùy chọn (Trống)", "✅ Đã khai tên - CV sẽ tự khớp theo tên")</f>
         <v/>
       </c>
     </row>
@@ -2162,7 +2161,7 @@
         </is>
       </c>
       <c r="F74">
-        <f>IF(ISBLANK(C74), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D74), ISBLANK(E74)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
+        <f>IF(ISBLANK(C74), "⚪ Tùy chọn (Trống)", "✅ Đã khai tên - CV sẽ tự khớp theo tên")</f>
         <v/>
       </c>
     </row>
@@ -2193,7 +2192,7 @@
         </is>
       </c>
       <c r="F75">
-        <f>IF(ISBLANK(C75), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D75), ISBLANK(E75)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
+        <f>IF(ISBLANK(C75), "⚪ Tùy chọn (Trống)", "✅ Đã khai tên - CV sẽ tự khớp theo tên")</f>
         <v/>
       </c>
     </row>
@@ -2224,7 +2223,7 @@
         </is>
       </c>
       <c r="F76">
-        <f>IF(ISBLANK(C76), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D76), ISBLANK(E76)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
+        <f>IF(ISBLANK(C76), "⚪ Tùy chọn (Trống)", "✅ Đã khai tên - CV sẽ tự khớp theo tên")</f>
         <v/>
       </c>
     </row>
@@ -2240,7 +2239,7 @@
         </is>
       </c>
       <c r="F77">
-        <f>IF(ISBLANK(C77), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D77), ISBLANK(E77)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
+        <f>IF(ISBLANK(C77), "⚪ Tùy chọn (Trống)", "✅ Đã khai tên - CV sẽ tự khớp theo tên")</f>
         <v/>
       </c>
     </row>
@@ -2256,7 +2255,7 @@
         </is>
       </c>
       <c r="F78">
-        <f>IF(ISBLANK(C78), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D78), ISBLANK(E78)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
+        <f>IF(ISBLANK(C78), "⚪ Tùy chọn (Trống)", "✅ Đã khai tên - CV sẽ tự khớp theo tên")</f>
         <v/>
       </c>
     </row>
@@ -3470,7 +3469,7 @@
       <c r="D69" s="3" t="n"/>
       <c r="E69" s="3" t="n"/>
       <c r="F69">
-        <f>IF(ISBLANK(C69), "❌ CHƯA ĐIỀN THÔNG TIN CNĐT (BÁO LỖI)", IF(OR(ISBLANK(D69), ISBLANK(E69)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV Mặc định Đạo đức"))</f>
+        <f>IF(ISBLANK(C69), "❌ CHƯA ĐIỀN THÔNG TIN CNĐT (BÁO LỖI)", "✅ Đã khai chủ nhiệm đề tài - CV sẽ tự khớp theo tên")</f>
         <v/>
       </c>
     </row>
@@ -3486,7 +3485,7 @@
         </is>
       </c>
       <c r="F70">
-        <f>IF(ISBLANK(C70), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D70), ISBLANK(E70)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
+        <f>IF(ISBLANK(C70), "⚪ Tùy chọn (Trống)", "✅ Đã khai tên - CV sẽ tự khớp theo tên")</f>
         <v/>
       </c>
     </row>
@@ -3502,7 +3501,7 @@
         </is>
       </c>
       <c r="F71">
-        <f>IF(ISBLANK(C71), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D71), ISBLANK(E71)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
+        <f>IF(ISBLANK(C71), "⚪ Tùy chọn (Trống)", "✅ Đã khai tên - CV sẽ tự khớp theo tên")</f>
         <v/>
       </c>
     </row>
@@ -3518,7 +3517,7 @@
         </is>
       </c>
       <c r="F72">
-        <f>IF(ISBLANK(C72), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D72), ISBLANK(E72)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
+        <f>IF(ISBLANK(C72), "⚪ Tùy chọn (Trống)", "✅ Đã khai tên - CV sẽ tự khớp theo tên")</f>
         <v/>
       </c>
     </row>
@@ -3534,7 +3533,7 @@
         </is>
       </c>
       <c r="F73">
-        <f>IF(ISBLANK(C73), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D73), ISBLANK(E73)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
+        <f>IF(ISBLANK(C73), "⚪ Tùy chọn (Trống)", "✅ Đã khai tên - CV sẽ tự khớp theo tên")</f>
         <v/>
       </c>
     </row>
@@ -3550,7 +3549,7 @@
         </is>
       </c>
       <c r="F74">
-        <f>IF(ISBLANK(C74), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D74), ISBLANK(E74)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
+        <f>IF(ISBLANK(C74), "⚪ Tùy chọn (Trống)", "✅ Đã khai tên - CV sẽ tự khớp theo tên")</f>
         <v/>
       </c>
     </row>
@@ -3566,7 +3565,7 @@
         </is>
       </c>
       <c r="F75">
-        <f>IF(ISBLANK(C75), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D75), ISBLANK(E75)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
+        <f>IF(ISBLANK(C75), "⚪ Tùy chọn (Trống)", "✅ Đã khai tên - CV sẽ tự khớp theo tên")</f>
         <v/>
       </c>
     </row>
@@ -3582,7 +3581,7 @@
         </is>
       </c>
       <c r="F76">
-        <f>IF(ISBLANK(C76), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D76), ISBLANK(E76)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
+        <f>IF(ISBLANK(C76), "⚪ Tùy chọn (Trống)", "✅ Đã khai tên - CV sẽ tự khớp theo tên")</f>
         <v/>
       </c>
     </row>
@@ -3598,7 +3597,7 @@
         </is>
       </c>
       <c r="F77">
-        <f>IF(ISBLANK(C77), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D77), ISBLANK(E77)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
+        <f>IF(ISBLANK(C77), "⚪ Tùy chọn (Trống)", "✅ Đã khai tên - CV sẽ tự khớp theo tên")</f>
         <v/>
       </c>
     </row>
@@ -3614,7 +3613,7 @@
         </is>
       </c>
       <c r="F78">
-        <f>IF(ISBLANK(C78), "⚪ Tùy chọn (Trống)", IF(OR(ISBLANK(D78), ISBLANK(E78)), "❌ BÁO LỖI: CHƯA CÓ FILE CV TRONG THƯ MỤC KIỂM TRA (VUI LÒNG BỔ SUNG)", "✅ Đã kiểm tra &amp; liên kết CV"))</f>
+        <f>IF(ISBLANK(C78), "⚪ Tùy chọn (Trống)", "✅ Đã khai tên - CV sẽ tự khớp theo tên")</f>
         <v/>
       </c>
     </row>
@@ -3623,10 +3622,7 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <dataValidations count="2">
-    <dataValidation sqref="E68 E69 E70 E71 E72 E73 E74 E75 E76 E77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>='_Lists'!$A$1:$A$6</formula1>
-    </dataValidation>
+  <dataValidations count="1">
     <dataValidation sqref="C7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"TVCT_ĐGHQ,TNLS"</formula1>
     </dataValidation>
@@ -3641,48 +3637,313 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Lý lịch khoa học - Trương Hồng Sơn.docx</t>
+          <t>ten</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>hoc_ham_hoc_vi</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>don_vi</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>dia_chi</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>sdt</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>cccd</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>mst</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>so_tk</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>ngan_hang</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TM-Gs. Nguyen Cong Khan.pdf</t>
+          <t>Trương Hồng Sơn</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TS.BS.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Viện trưởng - Viện Y học Ứng dụng VN</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TM-PGs. Hoang Thi Thanh.pdf</t>
+          <t>Lưu Liên Hương</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Thạc sĩ</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Trung tâm NCKH - Viện VIAM</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TM-PGs. Nguyen Quang Dung.pdf</t>
+          <t>Lê Việt Anh</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Thạc sĩ</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Trung tâm NCKH - Viện VIAM</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TM-PGs. Tran Quang Trung.pdf</t>
+          <t>Lê Minh Khánh</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Bác sĩ</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Phòng khám VIAM</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TM-Ts. Nguyen Hung Long.pdf</t>
+          <t>Nguyễn Công Khẩn</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>GS.TS.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Hội đồng Đạo đức Y sinh Quốc gia</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Nguyễn Xuân Ninh</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PGS.TS.BS.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Viện Y học Ứng dụng Việt Nam</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Lê Bạch Mai</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>PGS.TS.BS.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Nguyên Phó Viện trưởng Viện Dinh dưỡng QG</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Nguyễn Thị Lâm</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>PGS.TS.BS.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Nguyên Phó Viện trưởng Viện Dinh dưỡng QG</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Nguyễn Quang Dũng</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>PGS.TS.BS.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Bộ môn Dinh dưỡng - ĐH Y Hà Nội</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Hoàng Hà Linh</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Thạc sĩ</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Trung tâm NCKH - Viện VIAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Trương Phan Hồng Hà</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Thạc sĩ</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Viện Y học Ứng dụng Việt Nam</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Trần Quang Trung</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>PGS.TS.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Hiệp hội Sữa Việt Nam</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Phạm Văn Hoàn</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PGS.TS.</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Viện Y học Ứng dụng Việt Nam</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Ninh Thị Nhung</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>PGS.TS.</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Trường Đại học Y Dược Thái Bình</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Trần Văn Ơn</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>PGS.TS.</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Trường Đại học Dược Hà Nội</t>
         </is>
       </c>
     </row>
@@ -3697,327 +3958,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ten</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>hoc_ham_hoc_vi</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>don_vi</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>dia_chi</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>sdt</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>email</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>cccd</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>mst</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>so_tk</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>ngan_hang</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Trương Hồng Sơn</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>TS.BS.</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Viện trưởng - Viện Y học Ứng dụng VN</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Lưu Liên Hương</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Thạc sĩ</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Trung tâm NCKH - Viện VIAM</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Lê Việt Anh</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Thạc sĩ</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Trung tâm NCKH - Viện VIAM</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Lê Minh Khánh</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Bác sĩ</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Phòng khám VIAM</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Nguyễn Công Khẩn</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>GS.TS.</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Hội đồng Đạo đức Y sinh Quốc gia</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Nguyễn Xuân Ninh</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>PGS.TS.BS.</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Viện Y học Ứng dụng Việt Nam</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Lê Bạch Mai</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>PGS.TS.BS.</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Nguyên Phó Viện trưởng Viện Dinh dưỡng QG</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Nguyễn Thị Lâm</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>PGS.TS.BS.</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Nguyên Phó Viện trưởng Viện Dinh dưỡng QG</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Nguyễn Quang Dũng</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>PGS.TS.BS.</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Bộ môn Dinh dưỡng - ĐH Y Hà Nội</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Hoàng Hà Linh</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Thạc sĩ</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Trung tâm NCKH - Viện VIAM</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Trương Phan Hồng Hà</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Thạc sĩ</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Viện Y học Ứng dụng Việt Nam</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Trần Quang Trung</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>PGS.TS.</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Hiệp hội Sữa Việt Nam</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Phạm Văn Hoàn</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>PGS.TS.</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Viện Y học Ứng dụng Việt Nam</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Ninh Thị Nhung</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>PGS.TS.</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Trường Đại học Y Dược Thái Bình</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Trần Văn Ơn</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>PGS.TS.</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Trường Đại học Dược Hà Nội</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -4064,7 +4004,6 @@
           <t>raw</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>Tên đề tài</t>
@@ -4087,7 +4026,6 @@
           <t>raw</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>Năm thực hiện hồ sơ</t>
@@ -4110,7 +4048,6 @@
           <t>raw</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>Cơ quan chủ trì</t>
@@ -4133,7 +4070,6 @@
           <t>raw_or_placeholder</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>Cơ quan phối hợp</t>
@@ -4156,7 +4092,6 @@
           <t>person_ho_ten</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>Chủ nhiệm đề tài - có học hàm/học vị</t>
@@ -4179,7 +4114,6 @@
           <t>person_ten</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>Chủ nhiệm đề tài - chỉ tên</t>
@@ -4202,7 +4136,6 @@
           <t>person_ten</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>Đồng chủ nhiệm đề tài - chỉ tên</t>
@@ -4225,7 +4158,6 @@
           <t>person_ho_ten</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>Đồng chủ nhiệm đề tài - có học hàm/học vị</t>
@@ -4248,7 +4180,6 @@
           <t>person_ho_ten</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>Thư ký đề tài</t>
@@ -4271,7 +4202,6 @@
           <t>timeline_start</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>Mốc bắt đầu (MM/YYYY)</t>
@@ -4294,7 +4224,6 @@
           <t>timeline_end</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>Mốc kết thúc (MM/YYYY)</t>

</xml_diff>

<commit_message>
refactor: migrate token configuration to JSON and update template directory structure
</commit_message>
<xml_diff>
--- a/Form checklist hồ sơ dự án.xlsx
+++ b/Form checklist hồ sơ dự án.xlsx
@@ -9,7 +9,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đề tài - Bánh ăn dặm VIAM 2027" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đề tài - Mẫu trắng dự án mới" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_NhanSu" sheetId="3" state="hidden" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Tokens" sheetId="4" state="hidden" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -2083,21 +2082,6 @@
           <t>Hồ sơ Chuyên gia / Thành viên 4 (Tùy chọn)</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>Nguyễn Công Khẩn</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>Chuyên gia hội đồng</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>TM-Gs. Nguyen Cong Khan.pdf</t>
-        </is>
-      </c>
       <c r="F72">
         <f>IF(ISBLANK(C72), "⚪ Tùy chọn (Trống)", "✅ Đã khai tên - CV sẽ tự khớp theo tên")</f>
         <v/>
@@ -2114,21 +2098,6 @@
           <t>Hồ sơ Chuyên gia / Thành viên 5 (Tùy chọn)</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>Hoàng Thị Thanh</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>Chuyên gia hội đồng</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>TM-PGs. Hoang Thi Thanh.pdf</t>
-        </is>
-      </c>
       <c r="F73">
         <f>IF(ISBLANK(C73), "⚪ Tùy chọn (Trống)", "✅ Đã khai tên - CV sẽ tự khớp theo tên")</f>
         <v/>
@@ -2145,21 +2114,6 @@
           <t>Hồ sơ Chuyên gia / Thành viên 6 (Tùy chọn)</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>Nguyễn Quang Dũng</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>Chuyên gia hội đồng</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>TM-PGs. Nguyen Quang Dung.pdf</t>
-        </is>
-      </c>
       <c r="F74">
         <f>IF(ISBLANK(C74), "⚪ Tùy chọn (Trống)", "✅ Đã khai tên - CV sẽ tự khớp theo tên")</f>
         <v/>
@@ -2176,21 +2130,6 @@
           <t>Hồ sơ Chuyên gia / Thành viên 7 (Tùy chọn)</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>Trần Quang Trung</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>Chuyên gia hội đồng</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>TM-PGs. Tran Quang Trung.pdf</t>
-        </is>
-      </c>
       <c r="F75">
         <f>IF(ISBLANK(C75), "⚪ Tùy chọn (Trống)", "✅ Đã khai tên - CV sẽ tự khớp theo tên")</f>
         <v/>
@@ -2205,21 +2144,6 @@
       <c r="B76" t="inlineStr">
         <is>
           <t>Hồ sơ Chuyên gia / Thành viên 8 (Tùy chọn)</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>Nguyễn Hùng Long</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>Chuyên gia hội đồng</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>TM-Ts. Nguyen Hung Long.pdf</t>
         </is>
       </c>
       <c r="F76">
@@ -3950,341 +3874,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>token_name</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>kind</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>param</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>TEN_DE_TAI</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>A01</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>raw</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Tên đề tài</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>NAM</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>A03</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>raw</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Năm thực hiện hồ sơ</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>DON_VI_CHU_TRI</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>A04</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>raw</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Cơ quan chủ trì</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>DON_VI_DOI_TAC</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>A06</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>raw_or_placeholder</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Cơ quan phối hợp</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>CHU_NHIEM_HO_TEN</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>B01</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>person_ho_ten</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Chủ nhiệm đề tài - có học hàm/học vị</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>CHU_NHIEM_TEN</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>B01</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>person_ten</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Chủ nhiệm đề tài - chỉ tên</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>DONG_CHU_NHIEM_TEN</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>B02</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>person_ten</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Đồng chủ nhiệm đề tài - chỉ tên</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>DONG_CHU_NHIEM_HO_TEN</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>B02</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>person_ho_ten</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Đồng chủ nhiệm đề tài - có học hàm/học vị</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>THU_KY_DE_TAI</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>B03</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>person_ho_ten</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Thư ký đề tài</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>THOI_GIAN_BAT_DAU</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>A05</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>timeline_start</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Mốc bắt đầu (MM/YYYY)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>THOI_GIAN_KET_THUC</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>A05</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>timeline_end</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Mốc kết thúc (MM/YYYY)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>DIA_DIEM_TRIEN_KHAI</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>A07</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>raw_or_placeholder</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>……………………………</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Địa điểm triển khai nghiên cứu</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>DAU_MOI_LIEN_HE</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>A08</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>raw_or_placeholder</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>……</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Đầu mối liên hệ (thư mời chuyên gia)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: restructure project modules, migrate legacy scripts, and update template references and test suite.
</commit_message>
<xml_diff>
--- a/Form checklist hồ sơ dự án.xlsx
+++ b/Form checklist hồ sơ dự án.xlsx
@@ -9,6 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đề tài - Bánh ăn dặm VIAM 2027" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đề tài - Mẫu trắng dự án mới" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_NhanSu" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Tokens" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -17,8 +18,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="6">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
+  </numFmts>
+  <fonts count="8">
     <font>
       <name val="Arial"/>
       <family val="2"/>
@@ -61,8 +64,18 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F497D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -93,8 +106,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCE6F1"/>
+        <bgColor rgb="00DCE6F1"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -102,11 +121,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -114,6 +147,9 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -511,7 +547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F78"/>
+  <dimension ref="A1:F99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="8.5" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -535,6 +571,7 @@
         <v/>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -2183,11 +2220,423 @@
         <v/>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" s="7" t="inlineStr">
+        <is>
+          <t>SEC_G</t>
+        </is>
+      </c>
+      <c r="B79" s="7" t="inlineStr">
+        <is>
+          <t>PHẦN G: SỐ VĂN BẢN, NGÀY KÝ, BỐI CẢNH &amp; LỊCH HỌP (TÙY CHỌN - ĐỂ TRỐNG SẼ GIỮ NGUYÊN DẤU CHẤM LỬNG)</t>
+        </is>
+      </c>
+      <c r="C79" s="7" t="n"/>
+      <c r="D79" s="7" t="n"/>
+      <c r="E79" s="7" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="8" t="inlineStr">
+        <is>
+          <t>G01</t>
+        </is>
+      </c>
+      <c r="B80" s="8" t="inlineStr">
+        <is>
+          <t>Bối cảnh / lý do triển khai đề tài (Điền nội dung hoặc để trống)</t>
+        </is>
+      </c>
+      <c r="C80" s="8" t="n"/>
+      <c r="D80" s="8" t="inlineStr">
+        <is>
+          <t>Token: {{BOI_CANH_DU_AN}}</t>
+        </is>
+      </c>
+      <c r="E80" s="8" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="8" t="inlineStr">
+        <is>
+          <t>G02</t>
+        </is>
+      </c>
+      <c r="B81" s="8" t="inlineStr">
+        <is>
+          <t>Địa điểm họp Hội đồng (Tùy chọn - Để trống dùng địa chỉ Viện)</t>
+        </is>
+      </c>
+      <c r="C81" s="8" t="n"/>
+      <c r="D81" s="8" t="inlineStr">
+        <is>
+          <t>Token: {{DIA_DIEM_HOP}}</t>
+        </is>
+      </c>
+      <c r="E81" s="8" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="8" t="inlineStr">
+        <is>
+          <t>G03</t>
+        </is>
+      </c>
+      <c r="B82" s="8" t="inlineStr">
+        <is>
+          <t>Thời gian họp chung (giờ, ngày tháng - Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C82" s="8" t="n"/>
+      <c r="D82" s="8" t="inlineStr">
+        <is>
+          <t>Token: {{THOI_GIAN_HOP}}</t>
+        </is>
+      </c>
+      <c r="E82" s="8" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="8" t="inlineStr">
+        <is>
+          <t>G04</t>
+        </is>
+      </c>
+      <c r="B83" s="8" t="inlineStr">
+        <is>
+          <t>Số công văn mời chuyên gia (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C83" s="8" t="n"/>
+      <c r="D83" s="8" t="inlineStr">
+        <is>
+          <t>Token: {{SO_CONG_VAN}}</t>
+        </is>
+      </c>
+      <c r="E83" s="8" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="8" t="inlineStr">
+        <is>
+          <t>G05</t>
+        </is>
+      </c>
+      <c r="B84" s="8" t="inlineStr">
+        <is>
+          <t>Ngày ký công văn mời chuyên gia (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C84" s="9" t="n"/>
+      <c r="D84" s="8" t="inlineStr">
+        <is>
+          <t>Định dạng: DD/MM/YYYY</t>
+        </is>
+      </c>
+      <c r="E84" s="8" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="8" t="inlineStr">
+        <is>
+          <t>G06</t>
+        </is>
+      </c>
+      <c r="B85" s="8" t="inlineStr">
+        <is>
+          <t>Số Quyết định giao đề tài - Mẫu 00 (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="n"/>
+      <c r="D85" s="8" t="inlineStr">
+        <is>
+          <t>Token: {{SO_QD_GIAO_DE_TAI}}</t>
+        </is>
+      </c>
+      <c r="E85" s="8" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="8" t="inlineStr">
+        <is>
+          <t>G07</t>
+        </is>
+      </c>
+      <c r="B86" s="8" t="inlineStr">
+        <is>
+          <t>Ngày ký QĐ giao đề tài (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C86" s="9" t="n"/>
+      <c r="D86" s="8" t="inlineStr">
+        <is>
+          <t>Định dạng: DD/MM/YYYY</t>
+        </is>
+      </c>
+      <c r="E86" s="8" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="8" t="inlineStr">
+        <is>
+          <t>G08</t>
+        </is>
+      </c>
+      <c r="B87" s="8" t="inlineStr">
+        <is>
+          <t>Số QĐ TLHĐ Đạo đức - Mẫu 01 (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="n"/>
+      <c r="D87" s="8" t="inlineStr">
+        <is>
+          <t>Token: {{SO_QD_TLHD_DAO_DUC}}</t>
+        </is>
+      </c>
+      <c r="E87" s="8" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="8" t="inlineStr">
+        <is>
+          <t>G09</t>
+        </is>
+      </c>
+      <c r="B88" s="8" t="inlineStr">
+        <is>
+          <t>Ngày ký QĐ TLHĐ Đạo đức (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C88" s="9" t="n"/>
+      <c r="D88" s="8" t="inlineStr">
+        <is>
+          <t>Định dạng: DD/MM/YYYY</t>
+        </is>
+      </c>
+      <c r="E88" s="8" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="8" t="inlineStr">
+        <is>
+          <t>G10</t>
+        </is>
+      </c>
+      <c r="B89" s="8" t="inlineStr">
+        <is>
+          <t>Số QĐ TLHĐ Khoa học - Mẫu 05 (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C89" s="8" t="n"/>
+      <c r="D89" s="8" t="inlineStr">
+        <is>
+          <t>Token: {{SO_QD_TLHD_KHOA_HOC}}</t>
+        </is>
+      </c>
+      <c r="E89" s="8" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="8" t="inlineStr">
+        <is>
+          <t>G11</t>
+        </is>
+      </c>
+      <c r="B90" s="8" t="inlineStr">
+        <is>
+          <t>Ngày ký QĐ TLHĐ Khoa học (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C90" s="9" t="n"/>
+      <c r="D90" s="8" t="inlineStr">
+        <is>
+          <t>Định dạng: DD/MM/YYYY</t>
+        </is>
+      </c>
+      <c r="E90" s="8" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="8" t="inlineStr">
+        <is>
+          <t>G12</t>
+        </is>
+      </c>
+      <c r="B91" s="8" t="inlineStr">
+        <is>
+          <t>Số QĐ TLHĐ Nghiệm thu - Mẫu 9 (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C91" s="8" t="n"/>
+      <c r="D91" s="8" t="inlineStr">
+        <is>
+          <t>Token: {{SO_QD_TLHD_NGHIEM_THU}}</t>
+        </is>
+      </c>
+      <c r="E91" s="8" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="8" t="inlineStr">
+        <is>
+          <t>G13</t>
+        </is>
+      </c>
+      <c r="B92" s="8" t="inlineStr">
+        <is>
+          <t>Ngày ký QĐ TLHĐ Nghiệm thu (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C92" s="9" t="n"/>
+      <c r="D92" s="8" t="inlineStr">
+        <is>
+          <t>Định dạng: DD/MM/YYYY</t>
+        </is>
+      </c>
+      <c r="E92" s="8" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="8" t="inlineStr">
+        <is>
+          <t>G14</t>
+        </is>
+      </c>
+      <c r="B93" s="8" t="inlineStr">
+        <is>
+          <t>Số QĐ Phê duyệt đề tài - Mẫu 08 (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C93" s="8" t="n"/>
+      <c r="D93" s="8" t="inlineStr">
+        <is>
+          <t>Token: {{SO_QD_PHE_DUYET}}</t>
+        </is>
+      </c>
+      <c r="E93" s="8" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="8" t="inlineStr">
+        <is>
+          <t>G15</t>
+        </is>
+      </c>
+      <c r="B94" s="8" t="inlineStr">
+        <is>
+          <t>Ngày ký QĐ Phê duyệt đề tài (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C94" s="9" t="n"/>
+      <c r="D94" s="8" t="inlineStr">
+        <is>
+          <t>Định dạng: DD/MM/YYYY</t>
+        </is>
+      </c>
+      <c r="E94" s="8" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="8" t="inlineStr">
+        <is>
+          <t>G16</t>
+        </is>
+      </c>
+      <c r="B95" s="8" t="inlineStr">
+        <is>
+          <t>Số QĐ Công nhận kết quả - Mẫu 12 (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C95" s="8" t="n"/>
+      <c r="D95" s="8" t="inlineStr">
+        <is>
+          <t>Token: {{SO_QD_CONG_NHAN}}</t>
+        </is>
+      </c>
+      <c r="E95" s="8" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="8" t="inlineStr">
+        <is>
+          <t>G17</t>
+        </is>
+      </c>
+      <c r="B96" s="8" t="inlineStr">
+        <is>
+          <t>Ngày ký QĐ Công nhận kết quả (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C96" s="9" t="n"/>
+      <c r="D96" s="8" t="inlineStr">
+        <is>
+          <t>Định dạng: DD/MM/YYYY</t>
+        </is>
+      </c>
+      <c r="E96" s="8" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="8" t="inlineStr">
+        <is>
+          <t>G18</t>
+        </is>
+      </c>
+      <c r="B97" s="8" t="inlineStr">
+        <is>
+          <t>Ngày họp HĐ Đạo đức - Mẫu 02, 03 (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C97" s="9" t="n"/>
+      <c r="D97" s="8" t="inlineStr">
+        <is>
+          <t>Định dạng: DD/MM/YYYY</t>
+        </is>
+      </c>
+      <c r="E97" s="8" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="8" t="inlineStr">
+        <is>
+          <t>G19</t>
+        </is>
+      </c>
+      <c r="B98" s="8" t="inlineStr">
+        <is>
+          <t>Ngày họp HĐ Khoa học - Mẫu 06, 07 (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C98" s="9" t="n"/>
+      <c r="D98" s="8" t="inlineStr">
+        <is>
+          <t>Định dạng: DD/MM/YYYY</t>
+        </is>
+      </c>
+      <c r="E98" s="8" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="8" t="inlineStr">
+        <is>
+          <t>G20</t>
+        </is>
+      </c>
+      <c r="B99" s="8" t="inlineStr">
+        <is>
+          <t>Ngày họp HĐ Nghiệm thu - Mẫu 10, 11 (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C99" s="9" t="n"/>
+      <c r="D99" s="8" t="inlineStr">
+        <is>
+          <t>Định dạng: DD/MM/YYYY</t>
+        </is>
+      </c>
+      <c r="E99" s="8" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
+  <dataValidations count="5">
+    <dataValidation sqref="C15 C16 C17 C18 C19 C20 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C36 C37 C38 C39 C40 C41 C42 C43 C44 C45 C47 C48 C49 C50 C51 C52 C53 C54 C55 C56 C58 C59 C60 C61 C62 C63 C64 C65 C66 C67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>='_NhanSu'!$A$2:$A$16</formula1>
+    </dataValidation>
+    <dataValidation sqref="C7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Nghiên cứu can thiệp,Nghiên cứu quan sát,Thử nghiệm lâm sàng,Đánh giá hiệu quả công thức,Khác"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D36 D37 D38 D39 D40 D41 D42 D43 D44 D45 D47 D48 D49 D50 D51 D52 D53 D54 D55 D56 D58 D59 D60 D61 D62 D63 D64 D65 D66 D67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"GS.TS.,PGS.TS.,TS.,ThS.,BS.CKII,BS.CKI,BS.,CN.,DS."</formula1>
+    </dataValidation>
+    <dataValidation sqref="A6 A7 A8 A9 A10 A11 A12 A13 A15 A16 A17 A18 A19 A20 A21 A22 A23 A24 A25 A26 A27 A28 A29 A30 A31 A32 A33 A34 A36 A37 A38 A39 A40 A41 A42 A43 A44 A45 A47 A48 A49 A50 A51 A52 A53 A54 A55 A56 A58 A59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>='_Tokens'!$A$2:$A$38</formula1>
+    </dataValidation>
+    <dataValidation sqref="C84 C86 C88 C90 C92 C94 C96 C97 C98 C99" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Sai định dạng ngày" error="Vui lòng nhập ngày hợp lệ (VD: 15/03/2027 hoặc chọn từ lịch)" promptTitle="Nhập ngày" prompt="Định dạng ngày: DD/MM/YYYY" type="date" operator="greaterThanOrEqual">
+      <formula1>DATE(1900,1,1)</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2198,7 +2647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F78"/>
+  <dimension ref="A1:F99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="8.5" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2222,6 +2671,7 @@
         <v/>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -2450,8 +2900,8 @@
         </is>
       </c>
       <c r="C15" s="3" t="n"/>
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="n"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
       <c r="F15">
         <f>IF(ISBLANK(C15), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
@@ -2740,11 +3190,6 @@
           <t>Nghiên cứu viên 16</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>(Để trống tên theo quy định)</t>
-        </is>
-      </c>
       <c r="F33">
         <f>IF(ISBLANK(C33), "⚪ Tùy chọn (Trống)", "✅ Xong")</f>
         <v/>
@@ -2759,11 +3204,6 @@
       <c r="B34" t="inlineStr">
         <is>
           <t>Nghiên cứu viên 17</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>(Để trống tên theo quy định)</t>
         </is>
       </c>
       <c r="F34">
@@ -2799,8 +3239,8 @@
         </is>
       </c>
       <c r="C36" s="3" t="n"/>
-      <c r="D36" s="3" t="n"/>
-      <c r="E36" s="3" t="n"/>
+      <c r="D36" s="3" t="inlineStr"/>
+      <c r="E36" s="3" t="inlineStr"/>
       <c r="F36">
         <f>IF(ISBLANK(C36), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
@@ -2818,8 +3258,8 @@
         </is>
       </c>
       <c r="C37" s="3" t="n"/>
-      <c r="D37" s="3" t="n"/>
-      <c r="E37" s="3" t="n"/>
+      <c r="D37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr"/>
       <c r="F37">
         <f>IF(ISBLANK(C37), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
@@ -2837,8 +3277,8 @@
         </is>
       </c>
       <c r="C38" s="3" t="n"/>
-      <c r="D38" s="3" t="n"/>
-      <c r="E38" s="3" t="n"/>
+      <c r="D38" s="3" t="inlineStr"/>
+      <c r="E38" s="3" t="inlineStr"/>
       <c r="F38">
         <f>IF(ISBLANK(C38), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
@@ -2856,8 +3296,8 @@
         </is>
       </c>
       <c r="C39" s="3" t="n"/>
-      <c r="D39" s="3" t="n"/>
-      <c r="E39" s="3" t="n"/>
+      <c r="D39" s="3" t="inlineStr"/>
+      <c r="E39" s="3" t="inlineStr"/>
       <c r="F39">
         <f>IF(ISBLANK(C39), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
@@ -2875,8 +3315,8 @@
         </is>
       </c>
       <c r="C40" s="3" t="n"/>
-      <c r="D40" s="3" t="n"/>
-      <c r="E40" s="3" t="n"/>
+      <c r="D40" s="3" t="inlineStr"/>
+      <c r="E40" s="3" t="inlineStr"/>
       <c r="F40">
         <f>IF(ISBLANK(C40), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
@@ -2942,8 +3382,8 @@
         </is>
       </c>
       <c r="C44" s="3" t="n"/>
-      <c r="D44" s="3" t="n"/>
-      <c r="E44" s="3" t="n"/>
+      <c r="D44" s="3" t="inlineStr"/>
+      <c r="E44" s="3" t="inlineStr"/>
       <c r="F44">
         <f>IF(ISBLANK(C44), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
@@ -2961,8 +3401,8 @@
         </is>
       </c>
       <c r="C45" s="3" t="n"/>
-      <c r="D45" s="3" t="n"/>
-      <c r="E45" s="3" t="n"/>
+      <c r="D45" s="3" t="inlineStr"/>
+      <c r="E45" s="3" t="inlineStr"/>
       <c r="F45">
         <f>IF(ISBLANK(C45), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
@@ -2996,8 +3436,8 @@
         </is>
       </c>
       <c r="C47" s="3" t="n"/>
-      <c r="D47" s="3" t="n"/>
-      <c r="E47" s="3" t="n"/>
+      <c r="D47" s="3" t="inlineStr"/>
+      <c r="E47" s="3" t="inlineStr"/>
       <c r="F47">
         <f>IF(ISBLANK(C47), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
@@ -3015,8 +3455,8 @@
         </is>
       </c>
       <c r="C48" s="3" t="n"/>
-      <c r="D48" s="3" t="n"/>
-      <c r="E48" s="3" t="n"/>
+      <c r="D48" s="3" t="inlineStr"/>
+      <c r="E48" s="3" t="inlineStr"/>
       <c r="F48">
         <f>IF(ISBLANK(C48), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
@@ -3034,8 +3474,8 @@
         </is>
       </c>
       <c r="C49" s="3" t="n"/>
-      <c r="D49" s="3" t="n"/>
-      <c r="E49" s="3" t="n"/>
+      <c r="D49" s="3" t="inlineStr"/>
+      <c r="E49" s="3" t="inlineStr"/>
       <c r="F49">
         <f>IF(ISBLANK(C49), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
@@ -3053,8 +3493,8 @@
         </is>
       </c>
       <c r="C50" s="3" t="n"/>
-      <c r="D50" s="3" t="n"/>
-      <c r="E50" s="3" t="n"/>
+      <c r="D50" s="3" t="inlineStr"/>
+      <c r="E50" s="3" t="inlineStr"/>
       <c r="F50">
         <f>IF(ISBLANK(C50), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
@@ -3072,8 +3512,8 @@
         </is>
       </c>
       <c r="C51" s="3" t="n"/>
-      <c r="D51" s="3" t="n"/>
-      <c r="E51" s="3" t="n"/>
+      <c r="D51" s="3" t="inlineStr"/>
+      <c r="E51" s="3" t="inlineStr"/>
       <c r="F51">
         <f>IF(ISBLANK(C51), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
@@ -3139,8 +3579,8 @@
         </is>
       </c>
       <c r="C55" s="3" t="n"/>
-      <c r="D55" s="3" t="n"/>
-      <c r="E55" s="3" t="n"/>
+      <c r="D55" s="3" t="inlineStr"/>
+      <c r="E55" s="3" t="inlineStr"/>
       <c r="F55">
         <f>IF(ISBLANK(C55), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
@@ -3158,8 +3598,8 @@
         </is>
       </c>
       <c r="C56" s="3" t="n"/>
-      <c r="D56" s="3" t="n"/>
-      <c r="E56" s="3" t="n"/>
+      <c r="D56" s="3" t="inlineStr"/>
+      <c r="E56" s="3" t="inlineStr"/>
       <c r="F56">
         <f>IF(ISBLANK(C56), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
@@ -3193,8 +3633,8 @@
         </is>
       </c>
       <c r="C58" s="3" t="n"/>
-      <c r="D58" s="3" t="n"/>
-      <c r="E58" s="3" t="n"/>
+      <c r="D58" s="3" t="inlineStr"/>
+      <c r="E58" s="3" t="inlineStr"/>
       <c r="F58">
         <f>IF(ISBLANK(C58), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
@@ -3212,8 +3652,8 @@
         </is>
       </c>
       <c r="C59" s="3" t="n"/>
-      <c r="D59" s="3" t="n"/>
-      <c r="E59" s="3" t="n"/>
+      <c r="D59" s="3" t="inlineStr"/>
+      <c r="E59" s="3" t="inlineStr"/>
       <c r="F59">
         <f>IF(ISBLANK(C59), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
@@ -3231,8 +3671,8 @@
         </is>
       </c>
       <c r="C60" s="3" t="n"/>
-      <c r="D60" s="3" t="n"/>
-      <c r="E60" s="3" t="n"/>
+      <c r="D60" s="3" t="inlineStr"/>
+      <c r="E60" s="3" t="inlineStr"/>
       <c r="F60">
         <f>IF(ISBLANK(C60), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
@@ -3250,8 +3690,8 @@
         </is>
       </c>
       <c r="C61" s="3" t="n"/>
-      <c r="D61" s="3" t="n"/>
-      <c r="E61" s="3" t="n"/>
+      <c r="D61" s="3" t="inlineStr"/>
+      <c r="E61" s="3" t="inlineStr"/>
       <c r="F61">
         <f>IF(ISBLANK(C61), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
@@ -3269,8 +3709,8 @@
         </is>
       </c>
       <c r="C62" s="3" t="n"/>
-      <c r="D62" s="3" t="n"/>
-      <c r="E62" s="3" t="n"/>
+      <c r="D62" s="3" t="inlineStr"/>
+      <c r="E62" s="3" t="inlineStr"/>
       <c r="F62">
         <f>IF(ISBLANK(C62), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
@@ -3336,8 +3776,8 @@
         </is>
       </c>
       <c r="C66" s="3" t="n"/>
-      <c r="D66" s="3" t="n"/>
-      <c r="E66" s="3" t="n"/>
+      <c r="D66" s="3" t="inlineStr"/>
+      <c r="E66" s="3" t="inlineStr"/>
       <c r="F66">
         <f>IF(ISBLANK(C66), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
@@ -3355,8 +3795,8 @@
         </is>
       </c>
       <c r="C67" s="3" t="n"/>
-      <c r="D67" s="3" t="n"/>
-      <c r="E67" s="3" t="n"/>
+      <c r="D67" s="3" t="inlineStr"/>
+      <c r="E67" s="3" t="inlineStr"/>
       <c r="F67">
         <f>IF(ISBLANK(C67), "❌ CHƯA ĐIỀN (BÁO LỖI)", "✅ Xong")</f>
         <v/>
@@ -3541,14 +3981,421 @@
         <v/>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" s="7" t="inlineStr">
+        <is>
+          <t>SEC_G</t>
+        </is>
+      </c>
+      <c r="B79" s="7" t="inlineStr">
+        <is>
+          <t>PHẦN G: SỐ VĂN BẢN, NGÀY KÝ, BỐI CẢNH &amp; LỊCH HỌP (TÙY CHỌN - ĐỂ TRỐNG SẼ GIỮ NGUYÊN DẤU CHẤM LỬNG)</t>
+        </is>
+      </c>
+      <c r="C79" s="7" t="n"/>
+      <c r="D79" s="7" t="n"/>
+      <c r="E79" s="7" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="8" t="inlineStr">
+        <is>
+          <t>G01</t>
+        </is>
+      </c>
+      <c r="B80" s="8" t="inlineStr">
+        <is>
+          <t>Bối cảnh / lý do triển khai đề tài (Điền nội dung hoặc để trống)</t>
+        </is>
+      </c>
+      <c r="C80" s="8" t="n"/>
+      <c r="D80" s="8" t="inlineStr">
+        <is>
+          <t>Token: {{BOI_CANH_DU_AN}}</t>
+        </is>
+      </c>
+      <c r="E80" s="8" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="8" t="inlineStr">
+        <is>
+          <t>G02</t>
+        </is>
+      </c>
+      <c r="B81" s="8" t="inlineStr">
+        <is>
+          <t>Địa điểm họp Hội đồng (Tùy chọn - Để trống dùng địa chỉ Viện)</t>
+        </is>
+      </c>
+      <c r="C81" s="8" t="n"/>
+      <c r="D81" s="8" t="inlineStr">
+        <is>
+          <t>Token: {{DIA_DIEM_HOP}}</t>
+        </is>
+      </c>
+      <c r="E81" s="8" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="8" t="inlineStr">
+        <is>
+          <t>G03</t>
+        </is>
+      </c>
+      <c r="B82" s="8" t="inlineStr">
+        <is>
+          <t>Thời gian họp chung (giờ, ngày tháng - Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C82" s="8" t="n"/>
+      <c r="D82" s="8" t="inlineStr">
+        <is>
+          <t>Token: {{THOI_GIAN_HOP}}</t>
+        </is>
+      </c>
+      <c r="E82" s="8" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="8" t="inlineStr">
+        <is>
+          <t>G04</t>
+        </is>
+      </c>
+      <c r="B83" s="8" t="inlineStr">
+        <is>
+          <t>Số công văn mời chuyên gia (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C83" s="8" t="n"/>
+      <c r="D83" s="8" t="inlineStr">
+        <is>
+          <t>Token: {{SO_CONG_VAN}}</t>
+        </is>
+      </c>
+      <c r="E83" s="8" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="8" t="inlineStr">
+        <is>
+          <t>G05</t>
+        </is>
+      </c>
+      <c r="B84" s="8" t="inlineStr">
+        <is>
+          <t>Ngày ký công văn mời chuyên gia (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C84" s="9" t="n"/>
+      <c r="D84" s="8" t="inlineStr">
+        <is>
+          <t>Định dạng: DD/MM/YYYY</t>
+        </is>
+      </c>
+      <c r="E84" s="8" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="8" t="inlineStr">
+        <is>
+          <t>G06</t>
+        </is>
+      </c>
+      <c r="B85" s="8" t="inlineStr">
+        <is>
+          <t>Số Quyết định giao đề tài - Mẫu 00 (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="n"/>
+      <c r="D85" s="8" t="inlineStr">
+        <is>
+          <t>Token: {{SO_QD_GIAO_DE_TAI}}</t>
+        </is>
+      </c>
+      <c r="E85" s="8" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="8" t="inlineStr">
+        <is>
+          <t>G07</t>
+        </is>
+      </c>
+      <c r="B86" s="8" t="inlineStr">
+        <is>
+          <t>Ngày ký QĐ giao đề tài (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C86" s="9" t="n"/>
+      <c r="D86" s="8" t="inlineStr">
+        <is>
+          <t>Định dạng: DD/MM/YYYY</t>
+        </is>
+      </c>
+      <c r="E86" s="8" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="8" t="inlineStr">
+        <is>
+          <t>G08</t>
+        </is>
+      </c>
+      <c r="B87" s="8" t="inlineStr">
+        <is>
+          <t>Số QĐ TLHĐ Đạo đức - Mẫu 01 (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="n"/>
+      <c r="D87" s="8" t="inlineStr">
+        <is>
+          <t>Token: {{SO_QD_TLHD_DAO_DUC}}</t>
+        </is>
+      </c>
+      <c r="E87" s="8" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="8" t="inlineStr">
+        <is>
+          <t>G09</t>
+        </is>
+      </c>
+      <c r="B88" s="8" t="inlineStr">
+        <is>
+          <t>Ngày ký QĐ TLHĐ Đạo đức (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C88" s="9" t="n"/>
+      <c r="D88" s="8" t="inlineStr">
+        <is>
+          <t>Định dạng: DD/MM/YYYY</t>
+        </is>
+      </c>
+      <c r="E88" s="8" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="8" t="inlineStr">
+        <is>
+          <t>G10</t>
+        </is>
+      </c>
+      <c r="B89" s="8" t="inlineStr">
+        <is>
+          <t>Số QĐ TLHĐ Khoa học - Mẫu 05 (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C89" s="8" t="n"/>
+      <c r="D89" s="8" t="inlineStr">
+        <is>
+          <t>Token: {{SO_QD_TLHD_KHOA_HOC}}</t>
+        </is>
+      </c>
+      <c r="E89" s="8" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="8" t="inlineStr">
+        <is>
+          <t>G11</t>
+        </is>
+      </c>
+      <c r="B90" s="8" t="inlineStr">
+        <is>
+          <t>Ngày ký QĐ TLHĐ Khoa học (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C90" s="9" t="n"/>
+      <c r="D90" s="8" t="inlineStr">
+        <is>
+          <t>Định dạng: DD/MM/YYYY</t>
+        </is>
+      </c>
+      <c r="E90" s="8" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="8" t="inlineStr">
+        <is>
+          <t>G12</t>
+        </is>
+      </c>
+      <c r="B91" s="8" t="inlineStr">
+        <is>
+          <t>Số QĐ TLHĐ Nghiệm thu - Mẫu 9 (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C91" s="8" t="n"/>
+      <c r="D91" s="8" t="inlineStr">
+        <is>
+          <t>Token: {{SO_QD_TLHD_NGHIEM_THU}}</t>
+        </is>
+      </c>
+      <c r="E91" s="8" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="8" t="inlineStr">
+        <is>
+          <t>G13</t>
+        </is>
+      </c>
+      <c r="B92" s="8" t="inlineStr">
+        <is>
+          <t>Ngày ký QĐ TLHĐ Nghiệm thu (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C92" s="9" t="n"/>
+      <c r="D92" s="8" t="inlineStr">
+        <is>
+          <t>Định dạng: DD/MM/YYYY</t>
+        </is>
+      </c>
+      <c r="E92" s="8" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="8" t="inlineStr">
+        <is>
+          <t>G14</t>
+        </is>
+      </c>
+      <c r="B93" s="8" t="inlineStr">
+        <is>
+          <t>Số QĐ Phê duyệt đề tài - Mẫu 08 (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C93" s="8" t="n"/>
+      <c r="D93" s="8" t="inlineStr">
+        <is>
+          <t>Token: {{SO_QD_PHE_DUYET}}</t>
+        </is>
+      </c>
+      <c r="E93" s="8" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="8" t="inlineStr">
+        <is>
+          <t>G15</t>
+        </is>
+      </c>
+      <c r="B94" s="8" t="inlineStr">
+        <is>
+          <t>Ngày ký QĐ Phê duyệt đề tài (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C94" s="9" t="n"/>
+      <c r="D94" s="8" t="inlineStr">
+        <is>
+          <t>Định dạng: DD/MM/YYYY</t>
+        </is>
+      </c>
+      <c r="E94" s="8" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="8" t="inlineStr">
+        <is>
+          <t>G16</t>
+        </is>
+      </c>
+      <c r="B95" s="8" t="inlineStr">
+        <is>
+          <t>Số QĐ Công nhận kết quả - Mẫu 12 (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C95" s="8" t="n"/>
+      <c r="D95" s="8" t="inlineStr">
+        <is>
+          <t>Token: {{SO_QD_CONG_NHAN}}</t>
+        </is>
+      </c>
+      <c r="E95" s="8" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="8" t="inlineStr">
+        <is>
+          <t>G17</t>
+        </is>
+      </c>
+      <c r="B96" s="8" t="inlineStr">
+        <is>
+          <t>Ngày ký QĐ Công nhận kết quả (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C96" s="9" t="n"/>
+      <c r="D96" s="8" t="inlineStr">
+        <is>
+          <t>Định dạng: DD/MM/YYYY</t>
+        </is>
+      </c>
+      <c r="E96" s="8" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="8" t="inlineStr">
+        <is>
+          <t>G18</t>
+        </is>
+      </c>
+      <c r="B97" s="8" t="inlineStr">
+        <is>
+          <t>Ngày họp HĐ Đạo đức - Mẫu 02, 03 (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C97" s="9" t="n"/>
+      <c r="D97" s="8" t="inlineStr">
+        <is>
+          <t>Định dạng: DD/MM/YYYY</t>
+        </is>
+      </c>
+      <c r="E97" s="8" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="8" t="inlineStr">
+        <is>
+          <t>G19</t>
+        </is>
+      </c>
+      <c r="B98" s="8" t="inlineStr">
+        <is>
+          <t>Ngày họp HĐ Khoa học - Mẫu 06, 07 (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C98" s="9" t="n"/>
+      <c r="D98" s="8" t="inlineStr">
+        <is>
+          <t>Định dạng: DD/MM/YYYY</t>
+        </is>
+      </c>
+      <c r="E98" s="8" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="8" t="inlineStr">
+        <is>
+          <t>G20</t>
+        </is>
+      </c>
+      <c r="B99" s="8" t="inlineStr">
+        <is>
+          <t>Ngày họp HĐ Nghiệm thu - Mẫu 10, 11 (Tùy chọn)</t>
+        </is>
+      </c>
+      <c r="C99" s="9" t="n"/>
+      <c r="D99" s="8" t="inlineStr">
+        <is>
+          <t>Định dạng: DD/MM/YYYY</t>
+        </is>
+      </c>
+      <c r="E99" s="8" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="5">
+    <dataValidation sqref="C15 C16 C17 C18 C19 C20 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C36 C37 C38 C39 C40 C41 C42 C43 C44 C45 C47 C48 C49 C50 C51 C52 C53 C54 C55 C56 C58 C59 C60 C61 C62 C63 C64 C65 C66 C67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>='_NhanSu'!$A$2:$A$16</formula1>
+    </dataValidation>
     <dataValidation sqref="C7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"TVCT_ĐGHQ,TNLS"</formula1>
+      <formula1>"Nghiên cứu can thiệp,Nghiên cứu quan sát,Thử nghiệm lâm sàng,Đánh giá hiệu quả công thức,Khác"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D36 D37 D38 D39 D40 D41 D42 D43 D44 D45 D47 D48 D49 D50 D51 D52 D53 D54 D55 D56 D58 D59 D60 D61 D62 D63 D64 D65 D66 D67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"GS.TS.,PGS.TS.,TS.,ThS.,BS.CKII,BS.CKI,BS.,CN.,DS."</formula1>
+    </dataValidation>
+    <dataValidation sqref="A6 A7 A8 A9 A10 A11 A12 A13 A15 A16 A17 A18 A19 A20 A21 A22 A23 A24 A25 A26 A27 A28 A29 A30 A31 A32 A33 A34 A36 A37 A38 A39 A40 A41 A42 A43 A44 A45 A47 A48 A49 A50 A51 A52 A53 A54 A55 A56 A58 A59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>='_Tokens'!$A$2:$A$38</formula1>
+    </dataValidation>
+    <dataValidation sqref="C84 C86 C88 C90 C92 C94 C96 C97 C98 C99" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Sai định dạng ngày" error="Vui lòng nhập ngày hợp lệ (VD: 15/03/2027 hoặc chọn từ lịch)" promptTitle="Nhập ngày" prompt="Định dạng ngày: DD/MM/YYYY" type="date" operator="greaterThanOrEqual">
+      <formula1>DATE(1900,1,1)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3874,4 +4721,664 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TOKEN_TAG</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>MÃ_MỤC</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>MÔ_TẢ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>{{TEN_DE_TAI}}</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>A01</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Tên đề tài nghiên cứu</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>{{NAM}}</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>A03</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Năm thực hiện hồ sơ</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>{{DON_VI_CHU_TRI}}</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>A04</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Cơ quan chủ trì</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>{{DON_VI_DOI_TAC}}</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>A06</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Cơ quan phối hợp (tùy chọn)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>{{THOI_GIAN_BAT_DAU}}</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>A05</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Mốc thời gian bắt đầu (MM/YYYY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>{{THOI_GIAN_KET_THUC}}</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>A05</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Mốc thời gian kết thúc (MM/YYYY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>{{DIA_DIEM_TRIEN_KHAI}}</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>A07</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Địa điểm triển khai nghiên cứu</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>{{DAU_MOI_LIEN_HE}}</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>A08</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Đầu mối liên hệ thư mời</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>{{CHU_NHIEM_HO_TEN}}</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>B01</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Họ tên Chủ nhiệm đề tài</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>{{CHU_NHIEM_TEN}}</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>B01</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Tên riêng Chủ nhiệm đề tài</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>{{CHU_NHIEM_DON_VI}}</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>B01</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Đơn vị công tác Chủ nhiệm đề tài</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>{{DONG_CHU_NHIEM_HO_TEN}}</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>B02</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Họ tên Đồng chủ nhiệm đề tài</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>{{THU_KY_DE_TAI}}</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>B03</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Họ tên Thư ký đề tài</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>{{DANH_SACH_NGHIEN_CUU_VIEN}}</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>B04-B20</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Danh sách nghiên cứu viên</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>{{CHU_TICH_HD_DAO_DUC}}</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>C01</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Chủ tịch HĐ Đạo đức</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>{{CHU_TICH_HD_KHOA_HOC}}</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>D01</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Chủ tịch HĐ Khoa học</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>{{CHU_TICH_HD_NGHIEM_THU}}</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>E01</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Chủ tịch HĐ Nghiệm thu</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>{{BOI_CANH_DU_AN}}</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>G01</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Bối cảnh / lý do triển khai đề tài</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>{{DIA_DIEM_HOP}}</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>G02</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Địa điểm họp Hội đồng</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>{{THOI_GIAN_HOP}}</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>G03</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Thời gian họp Hội đồng (giờ, ngày tháng)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>{{SO_CONG_VAN}}</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>G04</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Số công văn mời chuyên gia</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>{{NGAY_CONG_VAN}}</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>G05</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Ngày ký công văn mời chuyên gia</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>{{SO_QD_GIAO_DE_TAI}}</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>G06</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Số Quyết định giao đề tài (00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>{{NGAY_QD_GIAO_DE_TAI}}</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>G07</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Ngày ký QĐ giao đề tài</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>{{SO_QD_TLHD_DAO_DUC}}</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>G08</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Số QĐ TLHĐ Đạo đức (01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>{{NGAY_QD_TLHD_DAO_DUC}}</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>G09</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Ngày ký QĐ TLHĐ Đạo đức</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>{{SO_QD_TLHD_KHOA_HOC}}</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>G10</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Số QĐ TLHĐ Khoa học (05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>{{NGAY_QD_TLHD_KHOA_HOC}}</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>G11</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Ngày ký QĐ TLHĐ Khoa học</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>{{SO_QD_TLHD_PHE_DUYET}}</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>G14</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Số QĐ Phê duyệt đề tài (08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>{{NGAY_QD_PHE_DUYET}}</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>G15</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Ngày ký QĐ Phê duyệt đề tài</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>{{SO_QD_TLHD_NGHIEM_THU}}</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>G12</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Số QĐ TLHĐ Nghiệm thu (9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>{{NGAY_QD_TLHD_NGHIEM_THU}}</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>G13</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Ngày ký QĐ TLHĐ Nghiệm thu</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>{{SO_QD_CONG_NHAN}}</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>G16</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Số QĐ Công nhận kết quả (12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>{{NGAY_QD_CONG_NHAN}}</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>G17</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Ngày ký QĐ Công nhận kết quả</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>{{NGAY_HOP_DAO_DUC}}</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>G18</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Ngày họp HĐ Đạo đức (02, 03)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>{{NGAY_HOP_KHOA_HOC}}</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>G19</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Ngày họp HĐ Khoa học (06, 07)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>{{NGAY_HOP_NGHIEM_THU}}</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>G20</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Ngày họp HĐ Nghiệm thu (10, 11)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>